<commit_message>
WIP skrining mandiri remaja
</commit_message>
<xml_diff>
--- a/dataset/remaja.xlsx
+++ b/dataset/remaja.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843BCCF8-6257-AF4F-9318-335C4395842A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA3E77F-3B6F-2943-A4FC-1F163F9C1532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,13 +75,21 @@
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
+            <color rgb="FF000000"/>
             <rFont val="Aptos Narrow"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Microsoft Office User:
-diisi jika pernah_kencing_manis Tidak</t>
+          <t xml:space="preserve">Microsoft Office User:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>diisi jika pernah_kencing_manis Tidak</t>
         </r>
       </text>
     </comment>
@@ -100,7 +108,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -115,7 +123,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="BK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -130,7 +138,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="BP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -145,7 +153,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -160,7 +168,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="CJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -175,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="DB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -195,7 +203,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="182">
   <si>
     <t>batas_awal</t>
   </si>
@@ -227,64 +235,16 @@
     <t>anggota_keluarga_diabetes</t>
   </si>
   <si>
-    <t>imunisasi_24_bulan</t>
-  </si>
-  <si>
-    <t>membawa_buku_imunisasi</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_hepatitis_b</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_bcg</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_opv</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_dpt</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_opv_2</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_pcv</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_rotavirus</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_dpt_2</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_opv_3</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_pcv_2</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_rotavirus_2</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_dpt_3</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_opv_4</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_rotavirus_3</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_ipv</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_campak</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_dpt_4</t>
-  </si>
-  <si>
-    <t>menerima_imunisasi_campak_2</t>
+    <t>malaria_1</t>
+  </si>
+  <si>
+    <t>malaria_2</t>
+  </si>
+  <si>
+    <t>malaria_3</t>
+  </si>
+  <si>
+    <t>malaria_4</t>
   </si>
   <si>
     <t>berat_badan</t>
@@ -602,9 +562,24 @@
     <t>status</t>
   </si>
   <si>
+    <t>2026-06-05</t>
+  </si>
+  <si>
+    <t>2026-06-11</t>
+  </si>
+  <si>
+    <t>ACH. BIMA FAIRUS</t>
+  </si>
+  <si>
     <t>Tidak</t>
   </si>
   <si>
+    <t>Ya</t>
+  </si>
+  <si>
+    <t>Sudah</t>
+  </si>
+  <si>
     <t>Berdiri</t>
   </si>
   <si>
@@ -614,15 +589,9 @@
     <t>Perkembangan sesuai usia</t>
   </si>
   <si>
-    <t>Ya</t>
-  </si>
-  <si>
     <t>Tidak batuk</t>
   </si>
   <si>
-    <t>Sudah</t>
-  </si>
-  <si>
     <t>Negatif</t>
   </si>
   <si>
@@ -746,35 +715,47 @@
     <t>Pernah didiagnosis tuberkulosis (TBC)</t>
   </si>
   <si>
-    <t>FAILED: name 'false' is not defined</t>
-  </si>
-  <si>
-    <t>ACH. BIMA FAIRUS</t>
-  </si>
-  <si>
-    <t>2026-06-05</t>
-  </si>
-  <si>
-    <t>2026-06-11</t>
-  </si>
-  <si>
-    <t>malaria_1</t>
-  </si>
-  <si>
-    <t>malaria_2</t>
-  </si>
-  <si>
-    <t>malaria_3</t>
-  </si>
-  <si>
-    <t>malaria_4</t>
+    <t>FAILED: Timeout 30000ms exceeded.</t>
+  </si>
+  <si>
+    <t>cemas_1</t>
+  </si>
+  <si>
+    <t>cemas_2</t>
+  </si>
+  <si>
+    <t>cemas_3</t>
+  </si>
+  <si>
+    <t>depresi_1</t>
+  </si>
+  <si>
+    <t>depresi_2</t>
+  </si>
+  <si>
+    <t>depresi_3</t>
+  </si>
+  <si>
+    <t>hepatitis_sd_1</t>
+  </si>
+  <si>
+    <t>hepatitis_sd_2</t>
+  </si>
+  <si>
+    <t>hepatitis_sd_3</t>
+  </si>
+  <si>
+    <t>hepatitis_sd_4</t>
+  </si>
+  <si>
+    <t>risiko_tb_anak</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -795,6 +776,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1178,7 +1165,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EI2"/>
+  <dimension ref="A1:EA2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1190,104 +1177,97 @@
     <col min="7" max="8" width="13.83203125" customWidth="1"/>
     <col min="9" max="9" width="21.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.83203125" customWidth="1"/>
-    <col min="13" max="13" width="29" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.83203125" customWidth="1"/>
-    <col min="15" max="15" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="23.83203125" customWidth="1"/>
-    <col min="19" max="19" width="27.1640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="27.1640625" customWidth="1"/>
-    <col min="22" max="22" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="29" bestFit="1" customWidth="1"/>
-    <col min="24" max="34" width="29" customWidth="1"/>
-    <col min="35" max="36" width="14.33203125" customWidth="1"/>
-    <col min="37" max="37" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19" bestFit="1" customWidth="1"/>
-    <col min="39" max="41" width="19" customWidth="1"/>
-    <col min="42" max="42" width="25" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="14.83203125" customWidth="1"/>
-    <col min="49" max="49" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="10" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="16" bestFit="1" customWidth="1"/>
-    <col min="53" max="54" width="13.6640625" customWidth="1"/>
-    <col min="55" max="55" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="56" max="57" width="13.6640625" customWidth="1"/>
-    <col min="58" max="58" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="59" max="63" width="22.5" customWidth="1"/>
-    <col min="64" max="64" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="65" max="68" width="22.5" customWidth="1"/>
-    <col min="69" max="69" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="22.83203125" customWidth="1"/>
-    <col min="74" max="74" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="16.1640625" customWidth="1"/>
-    <col min="76" max="76" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="78" max="79" width="12.33203125" customWidth="1"/>
-    <col min="80" max="80" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="14.1640625" customWidth="1"/>
-    <col min="82" max="82" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="23.6640625" customWidth="1"/>
-    <col min="85" max="85" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="12.83203125" customWidth="1"/>
-    <col min="91" max="91" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="17.5" customWidth="1"/>
-    <col min="94" max="94" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="13" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="98" max="100" width="19.5" customWidth="1"/>
-    <col min="101" max="101" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="9.83203125" customWidth="1"/>
-    <col min="103" max="103" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="104" max="107" width="11.5" customWidth="1"/>
-    <col min="108" max="108" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="9" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="18.1640625" customWidth="1"/>
-    <col min="115" max="115" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="117" max="119" width="8.33203125" customWidth="1"/>
-    <col min="120" max="120" width="22" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="14" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="14" customWidth="1"/>
-    <col min="125" max="125" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="18.1640625" customWidth="1"/>
-    <col min="128" max="128" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="131" max="133" width="18.1640625" customWidth="1"/>
-    <col min="134" max="134" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="35" bestFit="1" customWidth="1"/>
-    <col min="136" max="136" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="137" max="137" width="18.1640625" customWidth="1"/>
-    <col min="138" max="138" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="139" max="139" width="10.83203125" customWidth="1"/>
+    <col min="11" max="14" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="20" width="9" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="13" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="13" customWidth="1"/>
+    <col min="27" max="28" width="14.33203125" customWidth="1"/>
+    <col min="29" max="29" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="19" bestFit="1" customWidth="1"/>
+    <col min="31" max="33" width="19" customWidth="1"/>
+    <col min="34" max="34" width="25" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="14.83203125" customWidth="1"/>
+    <col min="41" max="41" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="10" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="16" bestFit="1" customWidth="1"/>
+    <col min="45" max="46" width="13.6640625" customWidth="1"/>
+    <col min="47" max="47" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="49" width="13.6640625" customWidth="1"/>
+    <col min="50" max="50" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="51" max="55" width="22.5" customWidth="1"/>
+    <col min="56" max="56" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="57" max="60" width="22.5" customWidth="1"/>
+    <col min="61" max="61" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="22.83203125" customWidth="1"/>
+    <col min="66" max="66" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="16.1640625" customWidth="1"/>
+    <col min="68" max="68" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="70" max="71" width="12.33203125" customWidth="1"/>
+    <col min="72" max="72" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="14.1640625" customWidth="1"/>
+    <col min="74" max="74" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="23.6640625" customWidth="1"/>
+    <col min="77" max="77" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="12.83203125" customWidth="1"/>
+    <col min="83" max="83" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="17.5" customWidth="1"/>
+    <col min="86" max="86" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="13" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="90" max="92" width="19.5" customWidth="1"/>
+    <col min="93" max="93" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="9.83203125" customWidth="1"/>
+    <col min="95" max="95" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="96" max="99" width="11.5" customWidth="1"/>
+    <col min="100" max="100" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="9" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="18.1640625" customWidth="1"/>
+    <col min="107" max="107" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="109" max="111" width="8.33203125" customWidth="1"/>
+    <col min="112" max="112" width="22" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="14" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="14" customWidth="1"/>
+    <col min="117" max="117" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="18.1640625" customWidth="1"/>
+    <col min="120" max="120" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="123" max="125" width="18.1640625" customWidth="1"/>
+    <col min="126" max="126" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="35" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="18.1640625" customWidth="1"/>
+    <col min="130" max="130" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:139" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:131" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1318,932 +1298,889 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="Z1" s="2"/>
+      <c r="AA1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="AB1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="AC1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="AD1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="AE1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="AF1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="AG1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="AH1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="AI1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AJ1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AK1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AL1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AM1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AN1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AO1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AP1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="AG1" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="AI1" t="s">
+      <c r="AQ1" t="s">
         <v>30</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AR1" t="s">
         <v>31</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AS1" t="s">
         <v>32</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AT1" t="s">
         <v>33</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AU1" t="s">
         <v>34</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AV1" t="s">
         <v>35</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AW1" t="s">
         <v>36</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AX1" t="s">
         <v>37</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AY1" t="s">
         <v>38</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AZ1" t="s">
         <v>39</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="BA1" t="s">
         <v>40</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="BB1" t="s">
         <v>41</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="BC1" t="s">
         <v>42</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BD1" t="s">
         <v>43</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BE1" t="s">
         <v>44</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BF1" t="s">
         <v>45</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BG1" t="s">
         <v>46</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BH1" t="s">
         <v>47</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BI1" t="s">
         <v>48</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BJ1" t="s">
         <v>49</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BK1" t="s">
         <v>50</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BL1" t="s">
         <v>51</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BM1" t="s">
         <v>52</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BN1" t="s">
         <v>53</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BO1" t="s">
         <v>54</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BP1" t="s">
         <v>55</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BQ1" t="s">
         <v>56</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BR1" t="s">
         <v>57</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BS1" t="s">
         <v>58</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BT1" t="s">
         <v>59</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BU1" t="s">
         <v>60</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BV1" t="s">
         <v>61</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BW1" t="s">
         <v>62</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BX1" t="s">
         <v>63</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BY1" t="s">
         <v>64</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BZ1" t="s">
         <v>65</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="CA1" t="s">
         <v>66</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="CB1" t="s">
         <v>67</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CC1" t="s">
         <v>68</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CD1" t="s">
         <v>69</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CE1" t="s">
         <v>70</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CF1" t="s">
         <v>71</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CG1" t="s">
         <v>72</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CH1" t="s">
         <v>73</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CI1" t="s">
         <v>74</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CJ1" t="s">
         <v>75</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CK1" t="s">
         <v>76</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CL1" t="s">
         <v>77</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CM1" t="s">
         <v>78</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CN1" t="s">
         <v>79</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CO1" t="s">
         <v>80</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CP1" t="s">
         <v>81</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CQ1" t="s">
         <v>82</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CR1" t="s">
         <v>83</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CS1" t="s">
         <v>84</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CT1" t="s">
         <v>85</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CU1" t="s">
         <v>86</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CV1" t="s">
         <v>87</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CW1" t="s">
         <v>88</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CX1" t="s">
         <v>89</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CY1" t="s">
         <v>90</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CZ1" t="s">
         <v>91</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="DA1" t="s">
         <v>92</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="DB1" t="s">
         <v>93</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="DC1" t="s">
         <v>94</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="DD1" t="s">
         <v>95</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="DE1" t="s">
         <v>96</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="DF1" t="s">
         <v>97</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="DG1" t="s">
         <v>98</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DH1" t="s">
         <v>99</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DI1" t="s">
         <v>100</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DJ1" t="s">
         <v>101</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DK1" t="s">
         <v>102</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DL1" t="s">
         <v>103</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DM1" t="s">
         <v>104</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DN1" t="s">
         <v>105</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DO1" t="s">
         <v>106</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DP1" t="s">
         <v>107</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DQ1" t="s">
         <v>108</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DR1" t="s">
         <v>109</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DS1" t="s">
         <v>110</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DT1" t="s">
         <v>111</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DU1" t="s">
         <v>112</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DV1" t="s">
         <v>113</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DW1" t="s">
         <v>114</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="DX1" t="s">
         <v>115</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="DY1" t="s">
         <v>116</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="DZ1" t="s">
         <v>117</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="EA1" t="s">
         <v>118</v>
       </c>
-      <c r="DT1" t="s">
+    </row>
+    <row r="2" spans="1:131" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="B2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="C2" t="s">
         <v>121</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="E2" t="s">
         <v>122</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="G2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H2" t="s">
+        <v>122</v>
+      </c>
+      <c r="I2" t="s">
+        <v>122</v>
+      </c>
+      <c r="J2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K2" t="s">
+        <v>122</v>
+      </c>
+      <c r="L2" t="s">
+        <v>122</v>
+      </c>
+      <c r="M2" t="s">
+        <v>122</v>
+      </c>
+      <c r="N2" t="s">
+        <v>122</v>
+      </c>
+      <c r="O2" t="s">
+        <v>122</v>
+      </c>
+      <c r="P2" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>122</v>
+      </c>
+      <c r="R2" t="s">
+        <v>122</v>
+      </c>
+      <c r="S2" t="s">
+        <v>122</v>
+      </c>
+      <c r="T2" t="s">
+        <v>122</v>
+      </c>
+      <c r="U2" t="s">
+        <v>122</v>
+      </c>
+      <c r="V2" t="s">
+        <v>122</v>
+      </c>
+      <c r="W2" t="s">
+        <v>122</v>
+      </c>
+      <c r="X2" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>128</v>
+      </c>
+      <c r="AA2">
+        <v>30</v>
+      </c>
+      <c r="AB2">
+        <v>100</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>126</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>127</v>
+      </c>
+      <c r="AF2" t="s">
         <v>123</v>
       </c>
-      <c r="DY1" t="s">
+      <c r="AG2">
+        <v>10</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>126</v>
+      </c>
+      <c r="AO2" t="s">
         <v>124</v>
       </c>
-      <c r="DZ1" t="s">
-        <v>125</v>
-      </c>
-      <c r="EA1" t="s">
+      <c r="AP2">
+        <v>2900</v>
+      </c>
+      <c r="AQ2">
+        <v>6000</v>
+      </c>
+      <c r="AR2">
+        <v>80</v>
+      </c>
+      <c r="AS2">
+        <v>90</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>129</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>129</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>129</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>129</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>123</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>123</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>122</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>130</v>
+      </c>
+      <c r="BF2">
+        <v>30122025</v>
+      </c>
+      <c r="BG2" t="s">
         <v>126</v>
       </c>
-      <c r="EB1" t="s">
-        <v>127</v>
-      </c>
-      <c r="EC1" t="s">
-        <v>128</v>
-      </c>
-      <c r="ED1" t="s">
-        <v>129</v>
-      </c>
-      <c r="EE1" t="s">
-        <v>130</v>
-      </c>
-      <c r="EF1" t="s">
+      <c r="BH2" t="s">
         <v>131</v>
       </c>
-      <c r="EG1" t="s">
+      <c r="BI2" t="s">
         <v>132</v>
       </c>
-      <c r="EH1" t="s">
+      <c r="BJ2" t="s">
         <v>133</v>
       </c>
-      <c r="EI1" t="s">
+      <c r="BK2" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:139" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="C2" t="s">
-        <v>184</v>
-      </c>
-      <c r="E2" t="s">
-        <v>135</v>
-      </c>
-      <c r="G2" t="s">
-        <v>135</v>
-      </c>
-      <c r="H2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I2" t="s">
-        <v>135</v>
-      </c>
-      <c r="J2" t="s">
-        <v>135</v>
-      </c>
-      <c r="K2" t="s">
-        <v>139</v>
-      </c>
-      <c r="L2" t="s">
-        <v>139</v>
-      </c>
-      <c r="M2" t="s">
-        <v>141</v>
-      </c>
-      <c r="N2" t="s">
-        <v>141</v>
-      </c>
-      <c r="O2" t="s">
-        <v>141</v>
-      </c>
-      <c r="P2" t="s">
-        <v>141</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>141</v>
-      </c>
-      <c r="R2" t="s">
-        <v>141</v>
-      </c>
-      <c r="S2" t="s">
-        <v>141</v>
-      </c>
-      <c r="T2" t="s">
-        <v>141</v>
-      </c>
-      <c r="U2" t="s">
-        <v>141</v>
-      </c>
-      <c r="V2" t="s">
-        <v>141</v>
-      </c>
-      <c r="W2" t="s">
-        <v>141</v>
-      </c>
-      <c r="X2" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>141</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>135</v>
-      </c>
-      <c r="AI2">
-        <v>30</v>
-      </c>
-      <c r="AJ2">
-        <v>100</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>136</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>137</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>138</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AO2">
-        <v>10</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>137</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AX2">
-        <v>2900</v>
-      </c>
-      <c r="AY2">
-        <v>6000</v>
-      </c>
-      <c r="AZ2">
-        <v>80</v>
-      </c>
-      <c r="BA2">
-        <v>90</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>139</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>139</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>139</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>139</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>142</v>
       </c>
       <c r="BL2" t="s">
         <v>135</v>
       </c>
       <c r="BM2" t="s">
-        <v>143</v>
-      </c>
-      <c r="BN2">
-        <v>30122025</v>
+        <v>136</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>132</v>
       </c>
       <c r="BO2" t="s">
         <v>137</v>
       </c>
       <c r="BP2" t="s">
+        <v>138</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>132</v>
+      </c>
+      <c r="BR2" t="s">
+        <v>139</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>140</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>132</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>141</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>132</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>142</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>143</v>
+      </c>
+      <c r="BY2" t="s">
         <v>144</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BZ2" t="s">
+        <v>126</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>126</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CC2" t="s">
         <v>145</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="CD2" t="s">
+        <v>122</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CF2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CG2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CH2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CI2" t="s">
         <v>146</v>
       </c>
-      <c r="BS2" t="s">
+      <c r="CJ2" t="s">
         <v>147</v>
       </c>
-      <c r="BT2" t="s">
+      <c r="CK2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CL2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CM2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CN2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CP2" t="s">
         <v>148</v>
       </c>
-      <c r="BU2" t="s">
+      <c r="CQ2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CR2" t="s">
         <v>149</v>
       </c>
-      <c r="BV2" t="s">
-        <v>145</v>
-      </c>
-      <c r="BW2" t="s">
+      <c r="CS2" t="s">
+        <v>149</v>
+      </c>
+      <c r="CT2" t="s">
         <v>150</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="CU2" t="s">
         <v>151</v>
       </c>
-      <c r="BY2" t="s">
-        <v>145</v>
-      </c>
-      <c r="BZ2" t="s">
+      <c r="CV2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CW2" t="s">
         <v>152</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CX2" t="s">
         <v>153</v>
       </c>
-      <c r="CB2" t="s">
-        <v>145</v>
-      </c>
-      <c r="CC2" t="s">
+      <c r="CY2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CZ2" t="s">
         <v>154</v>
       </c>
-      <c r="CD2" t="s">
-        <v>145</v>
-      </c>
-      <c r="CE2" t="s">
+      <c r="DA2" t="s">
         <v>155</v>
       </c>
-      <c r="CF2" t="s">
+      <c r="DB2" t="s">
         <v>156</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="DC2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DD2" t="s">
         <v>157</v>
       </c>
-      <c r="CH2" t="s">
-        <v>137</v>
-      </c>
-      <c r="CI2" t="s">
-        <v>137</v>
-      </c>
-      <c r="CJ2" t="s">
-        <v>145</v>
-      </c>
-      <c r="CK2" t="s">
+      <c r="DE2" t="s">
+        <v>149</v>
+      </c>
+      <c r="DF2" t="s">
+        <v>148</v>
+      </c>
+      <c r="DG2" t="s">
         <v>158</v>
       </c>
-      <c r="CL2" t="s">
-        <v>135</v>
-      </c>
-      <c r="CM2" t="s">
-        <v>145</v>
-      </c>
-      <c r="CN2" t="s">
-        <v>139</v>
-      </c>
-      <c r="CO2" t="s">
-        <v>139</v>
-      </c>
-      <c r="CP2" t="s">
-        <v>145</v>
-      </c>
-      <c r="CQ2" t="s">
+      <c r="DH2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DI2" t="s">
+        <v>158</v>
+      </c>
+      <c r="DJ2" t="s">
         <v>159</v>
       </c>
-      <c r="CR2" t="s">
+      <c r="DK2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DL2" t="s">
+        <v>126</v>
+      </c>
+      <c r="DM2" t="s">
         <v>160</v>
       </c>
-      <c r="CS2" t="s">
-        <v>139</v>
-      </c>
-      <c r="CT2" t="s">
-        <v>139</v>
-      </c>
-      <c r="CU2" t="s">
-        <v>139</v>
-      </c>
-      <c r="CV2" t="s">
-        <v>139</v>
-      </c>
-      <c r="CW2" t="s">
-        <v>145</v>
-      </c>
-      <c r="CX2" t="s">
+      <c r="DN2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DO2" t="s">
         <v>161</v>
       </c>
-      <c r="CY2" t="s">
-        <v>145</v>
-      </c>
-      <c r="CZ2" t="s">
+      <c r="DP2" t="s">
         <v>162</v>
       </c>
-      <c r="DA2" t="s">
-        <v>162</v>
-      </c>
-      <c r="DB2" t="s">
+      <c r="DQ2" t="s">
+        <v>129</v>
+      </c>
+      <c r="DR2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DS2" t="s">
         <v>163</v>
       </c>
-      <c r="DC2" t="s">
+      <c r="DT2" t="s">
         <v>164</v>
       </c>
-      <c r="DD2" t="s">
-        <v>145</v>
-      </c>
-      <c r="DE2" t="s">
+      <c r="DU2" t="s">
         <v>165</v>
       </c>
-      <c r="DF2" t="s">
+      <c r="DV2" t="s">
         <v>166</v>
       </c>
-      <c r="DG2" t="s">
-        <v>145</v>
-      </c>
-      <c r="DH2" t="s">
+      <c r="DW2" t="s">
         <v>167</v>
       </c>
-      <c r="DI2" t="s">
+      <c r="DX2" t="s">
         <v>168</v>
       </c>
-      <c r="DJ2" t="s">
+      <c r="DY2" t="s">
         <v>169</v>
       </c>
-      <c r="DK2" t="s">
-        <v>145</v>
-      </c>
-      <c r="DL2" t="s">
+      <c r="DZ2" t="s">
+        <v>126</v>
+      </c>
+      <c r="EA2" t="s">
         <v>170</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>162</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>161</v>
-      </c>
-      <c r="DO2" t="s">
-        <v>171</v>
-      </c>
-      <c r="DP2" t="s">
-        <v>145</v>
-      </c>
-      <c r="DQ2" t="s">
-        <v>171</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>172</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>145</v>
-      </c>
-      <c r="DT2" t="s">
-        <v>137</v>
-      </c>
-      <c r="DU2" t="s">
-        <v>173</v>
-      </c>
-      <c r="DV2" t="s">
-        <v>145</v>
-      </c>
-      <c r="DW2" t="s">
-        <v>174</v>
-      </c>
-      <c r="DX2" t="s">
-        <v>175</v>
-      </c>
-      <c r="DY2" t="s">
-        <v>142</v>
-      </c>
-      <c r="DZ2" t="s">
-        <v>145</v>
-      </c>
-      <c r="EA2" t="s">
-        <v>176</v>
-      </c>
-      <c r="EB2" t="s">
-        <v>177</v>
-      </c>
-      <c r="EC2" t="s">
-        <v>178</v>
-      </c>
-      <c r="ED2" t="s">
-        <v>179</v>
-      </c>
-      <c r="EE2" t="s">
-        <v>180</v>
-      </c>
-      <c r="EF2" t="s">
-        <v>181</v>
-      </c>
-      <c r="EG2" t="s">
-        <v>182</v>
-      </c>
-      <c r="EH2" t="s">
-        <v>137</v>
-      </c>
-      <c r="EI2" t="s">
-        <v>183</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="42">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2:CV2 AN2 AQ2:AU2 BB2 BF2 BH2 BJ2 BL2 CL2 CN2:CO2 E2 K2:L2 AE2:AH2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="43">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 CK2:CN2 AF2 AI2:AM2 AT2 AX2 AZ2 BB2 BD2 CD2 CF2:CG2 K2:X2 Z2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2 ED2 EG2 BU2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2 BV2 BY2 CB2 CD2 CJ2 CM2 CP2 CW2 CY2 DD2 DG2 DK2 DP2 DS2 DV2 DZ2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2 BM2 DV2 DY2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2 BN2 BQ2 BT2 BV2 CB2 CE2 CH2 CO2 CQ2 CV2 CY2 DC2 DH2 DK2 DN2 DR2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2 G2:J2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J2 CI2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DB2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DW2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DO2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DP2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EE2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DW2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EH2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Berdiri,Telentang"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AD2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2 M2:AD2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BC2:BE2 BG2 BI2 BK2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AW2 AY2 BA2 BC2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2" xr:uid="{A76BCFDA-99B4-BC4C-9EB2-288C4CC41003}">
+      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="x12ac">
+          <x12ac:list>"Ya, lebih dari 2 minggu","Ya, kurang dari 2 minggu",Tidak batuk</x12ac:list>
+        </mc:Choice>
+        <mc:Fallback>
+          <formula1>"Ya, lebih dari 2 minggu,Ya, kurang dari 2 minggu,Tidak batuk"</formula1>
+        </mc:Fallback>
+      </mc:AlternateContent>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
wip gizi anak sekolah, tekanan darah dan gula darah
</commit_message>
<xml_diff>
--- a/dataset/remaja.xlsx
+++ b/dataset/remaja.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA3E77F-3B6F-2943-A4FC-1F163F9C1532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161121ED-0670-BD4F-A8AF-B74F5709EE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -108,7 +108,40 @@
         </r>
       </text>
     </comment>
-    <comment ref="AN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AF1" authorId="0" shapeId="0" xr:uid="{E74019AA-4207-6149-B0D4-EB4F1E6D6650}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>diisi jika anak_pernah_diabetes Ya</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -123,7 +156,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="BQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -138,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="BV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -153,7 +186,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="BY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -168,7 +201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="CP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -183,7 +216,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="DH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -203,7 +236,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="186">
   <si>
     <t>batas_awal</t>
   </si>
@@ -749,13 +782,25 @@
   </si>
   <si>
     <t>risiko_tb_anak</t>
+  </si>
+  <si>
+    <t>sistol</t>
+  </si>
+  <si>
+    <t>diastol</t>
+  </si>
+  <si>
+    <t>anak_pernah_diabetes</t>
+  </si>
+  <si>
+    <t>gds</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -781,6 +826,19 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1165,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EA2"/>
+  <dimension ref="A1:EG2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1182,92 +1240,92 @@
     <col min="18" max="20" width="9" bestFit="1" customWidth="1"/>
     <col min="21" max="24" width="13" bestFit="1" customWidth="1"/>
     <col min="25" max="26" width="13" customWidth="1"/>
-    <col min="27" max="28" width="14.33203125" customWidth="1"/>
-    <col min="29" max="29" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="19" bestFit="1" customWidth="1"/>
-    <col min="31" max="33" width="19" customWidth="1"/>
-    <col min="34" max="34" width="25" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="14.83203125" customWidth="1"/>
-    <col min="41" max="41" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="10" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="16" bestFit="1" customWidth="1"/>
-    <col min="45" max="46" width="13.6640625" customWidth="1"/>
-    <col min="47" max="47" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="48" max="49" width="13.6640625" customWidth="1"/>
-    <col min="50" max="50" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="51" max="55" width="22.5" customWidth="1"/>
-    <col min="56" max="56" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="57" max="60" width="22.5" customWidth="1"/>
-    <col min="61" max="61" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="22.83203125" customWidth="1"/>
-    <col min="66" max="66" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="16.1640625" customWidth="1"/>
-    <col min="68" max="68" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="70" max="71" width="12.33203125" customWidth="1"/>
-    <col min="72" max="72" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="14.1640625" customWidth="1"/>
-    <col min="74" max="74" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="23.6640625" customWidth="1"/>
-    <col min="77" max="77" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="12.83203125" customWidth="1"/>
-    <col min="83" max="83" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="17.5" customWidth="1"/>
-    <col min="86" max="86" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="13" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="90" max="92" width="19.5" customWidth="1"/>
-    <col min="93" max="93" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="9.83203125" customWidth="1"/>
-    <col min="95" max="95" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="96" max="99" width="11.5" customWidth="1"/>
-    <col min="100" max="100" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="9" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="18.1640625" customWidth="1"/>
-    <col min="107" max="107" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="109" max="111" width="8.33203125" customWidth="1"/>
-    <col min="112" max="112" width="22" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="14" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="14" customWidth="1"/>
-    <col min="117" max="117" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="18.1640625" customWidth="1"/>
-    <col min="120" max="120" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="123" max="125" width="18.1640625" customWidth="1"/>
-    <col min="126" max="126" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="35" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="18.1640625" customWidth="1"/>
-    <col min="130" max="130" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="10.83203125" customWidth="1"/>
+    <col min="27" max="34" width="14.33203125" customWidth="1"/>
+    <col min="35" max="35" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="19" bestFit="1" customWidth="1"/>
+    <col min="37" max="39" width="19" customWidth="1"/>
+    <col min="40" max="40" width="25" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="14.83203125" customWidth="1"/>
+    <col min="47" max="47" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="10" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="16" bestFit="1" customWidth="1"/>
+    <col min="51" max="52" width="13.6640625" customWidth="1"/>
+    <col min="53" max="53" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="54" max="55" width="13.6640625" customWidth="1"/>
+    <col min="56" max="56" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="57" max="61" width="22.5" customWidth="1"/>
+    <col min="62" max="62" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="66" width="22.5" customWidth="1"/>
+    <col min="67" max="67" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="22.83203125" customWidth="1"/>
+    <col min="72" max="72" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="16.1640625" customWidth="1"/>
+    <col min="74" max="74" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="76" max="77" width="12.33203125" customWidth="1"/>
+    <col min="78" max="78" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="14.1640625" customWidth="1"/>
+    <col min="80" max="80" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="23.6640625" customWidth="1"/>
+    <col min="83" max="83" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="12.83203125" customWidth="1"/>
+    <col min="89" max="89" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="17.5" customWidth="1"/>
+    <col min="92" max="92" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="13" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="96" max="98" width="19.5" customWidth="1"/>
+    <col min="99" max="99" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="9.83203125" customWidth="1"/>
+    <col min="101" max="101" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="102" max="105" width="11.5" customWidth="1"/>
+    <col min="106" max="106" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="9" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="18.1640625" customWidth="1"/>
+    <col min="113" max="113" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="115" max="117" width="8.33203125" customWidth="1"/>
+    <col min="118" max="118" width="22" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="14" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="14" customWidth="1"/>
+    <col min="123" max="123" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="18.1640625" customWidth="1"/>
+    <col min="126" max="126" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="129" max="131" width="18.1640625" customWidth="1"/>
+    <col min="132" max="132" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="133" max="133" width="35" bestFit="1" customWidth="1"/>
+    <col min="134" max="134" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="135" max="135" width="18.1640625" customWidth="1"/>
+    <col min="136" max="136" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="137" max="137" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:131" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:137" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1350,317 +1408,333 @@
       <c r="AB1" t="s">
         <v>15</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="AH1" s="2"/>
+      <c r="AI1" t="s">
         <v>16</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AJ1" t="s">
         <v>17</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AK1" t="s">
         <v>18</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AL1" t="s">
         <v>19</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AM1" t="s">
         <v>20</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AN1" t="s">
         <v>21</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AO1" t="s">
         <v>22</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AP1" t="s">
         <v>23</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AQ1" t="s">
         <v>24</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AR1" t="s">
         <v>25</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AS1" t="s">
         <v>26</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AT1" t="s">
         <v>27</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AU1" t="s">
         <v>28</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AV1" t="s">
         <v>29</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AW1" t="s">
         <v>30</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AX1" t="s">
         <v>31</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AY1" t="s">
         <v>32</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AZ1" t="s">
         <v>33</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="BA1" t="s">
         <v>34</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BB1" t="s">
         <v>35</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BC1" t="s">
         <v>36</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BD1" t="s">
         <v>37</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BE1" t="s">
         <v>38</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BF1" t="s">
         <v>39</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BG1" t="s">
         <v>40</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BH1" t="s">
         <v>41</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BI1" t="s">
         <v>42</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BJ1" t="s">
         <v>43</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BK1" t="s">
         <v>44</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BL1" t="s">
         <v>45</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BM1" t="s">
         <v>46</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BN1" t="s">
         <v>47</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BO1" t="s">
         <v>48</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BP1" t="s">
         <v>49</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BQ1" t="s">
         <v>50</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BR1" t="s">
         <v>51</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BS1" t="s">
         <v>52</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BT1" t="s">
         <v>53</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BU1" t="s">
         <v>54</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BV1" t="s">
         <v>55</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BW1" t="s">
         <v>56</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BX1" t="s">
         <v>57</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BY1" t="s">
         <v>58</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BZ1" t="s">
         <v>59</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CA1" t="s">
         <v>60</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CB1" t="s">
         <v>61</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CC1" t="s">
         <v>62</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CD1" t="s">
         <v>63</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CE1" t="s">
         <v>64</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CF1" t="s">
         <v>65</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CG1" t="s">
         <v>66</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CH1" t="s">
         <v>67</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CI1" t="s">
         <v>68</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CJ1" t="s">
         <v>69</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CK1" t="s">
         <v>70</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CL1" t="s">
         <v>71</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CM1" t="s">
         <v>72</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CN1" t="s">
         <v>73</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CO1" t="s">
         <v>74</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CP1" t="s">
         <v>75</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CQ1" t="s">
         <v>76</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CR1" t="s">
         <v>77</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CS1" t="s">
         <v>78</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CT1" t="s">
         <v>79</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CU1" t="s">
         <v>80</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CV1" t="s">
         <v>81</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CW1" t="s">
         <v>82</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CX1" t="s">
         <v>83</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CY1" t="s">
         <v>84</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CZ1" t="s">
         <v>85</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="DA1" t="s">
         <v>86</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="DB1" t="s">
         <v>87</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="DC1" t="s">
         <v>88</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="DD1" t="s">
         <v>89</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="DE1" t="s">
         <v>90</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DF1" t="s">
         <v>91</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DG1" t="s">
         <v>92</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DH1" t="s">
         <v>93</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DI1" t="s">
         <v>94</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DJ1" t="s">
         <v>95</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DK1" t="s">
         <v>96</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DL1" t="s">
         <v>97</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DM1" t="s">
         <v>98</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DN1" t="s">
         <v>99</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DO1" t="s">
         <v>100</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DP1" t="s">
         <v>101</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DQ1" t="s">
         <v>102</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DR1" t="s">
         <v>103</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DS1" t="s">
         <v>104</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DT1" t="s">
         <v>105</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DU1" t="s">
         <v>106</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="DV1" t="s">
         <v>107</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="DW1" t="s">
         <v>108</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="DX1" t="s">
         <v>109</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="DY1" t="s">
         <v>110</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="DZ1" t="s">
         <v>111</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="EA1" t="s">
         <v>112</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="EB1" t="s">
         <v>113</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="EC1" t="s">
         <v>114</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="ED1" t="s">
         <v>115</v>
       </c>
-      <c r="DY1" t="s">
+      <c r="EE1" t="s">
         <v>116</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="EF1" t="s">
         <v>117</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="EG1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:131" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:137" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>119</v>
       </c>
@@ -1731,79 +1805,73 @@
         <v>128</v>
       </c>
       <c r="AA2">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="AB2">
-        <v>100</v>
-      </c>
-      <c r="AC2" t="s">
+        <v>130</v>
+      </c>
+      <c r="AC2">
+        <v>120</v>
+      </c>
+      <c r="AD2">
+        <v>80</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>122</v>
+      </c>
+      <c r="AG2">
+        <v>120</v>
+      </c>
+      <c r="AI2" t="s">
         <v>125</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AJ2" t="s">
         <v>126</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AK2" t="s">
         <v>127</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AG2">
-        <v>10</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>128</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>123</v>
       </c>
       <c r="AL2" t="s">
         <v>123</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AM2">
+        <v>10</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>128</v>
+      </c>
+      <c r="AO2" t="s">
         <v>123</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AP2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>123</v>
+      </c>
+      <c r="AT2" t="s">
         <v>126</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AU2" t="s">
         <v>124</v>
       </c>
-      <c r="AP2">
+      <c r="AV2">
         <v>2900</v>
       </c>
-      <c r="AQ2">
+      <c r="AW2">
         <v>6000</v>
       </c>
-      <c r="AR2">
+      <c r="AX2">
         <v>80</v>
       </c>
-      <c r="AS2">
+      <c r="AY2">
         <v>90</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>129</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>129</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>129</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>129</v>
       </c>
       <c r="AZ2" t="s">
         <v>123</v>
@@ -1812,112 +1880,112 @@
         <v>129</v>
       </c>
       <c r="BB2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="BC2" t="s">
         <v>129</v>
       </c>
       <c r="BD2" t="s">
+        <v>123</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BF2" t="s">
+        <v>123</v>
+      </c>
+      <c r="BG2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>123</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BJ2" t="s">
         <v>122</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BK2" t="s">
         <v>130</v>
       </c>
-      <c r="BF2">
+      <c r="BL2">
         <v>30122025</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BM2" t="s">
         <v>126</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BN2" t="s">
         <v>131</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BO2" t="s">
         <v>132</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BP2" t="s">
         <v>133</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BQ2" t="s">
         <v>134</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BR2" t="s">
         <v>135</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BS2" t="s">
         <v>136</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>132</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>137</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>138</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>132</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>139</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>140</v>
       </c>
       <c r="BT2" t="s">
         <v>132</v>
       </c>
       <c r="BU2" t="s">
+        <v>137</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>138</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>132</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>139</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>140</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CA2" t="s">
         <v>141</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>132</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>142</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>143</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>144</v>
-      </c>
-      <c r="BZ2" t="s">
-        <v>126</v>
-      </c>
-      <c r="CA2" t="s">
-        <v>126</v>
       </c>
       <c r="CB2" t="s">
         <v>132</v>
       </c>
       <c r="CC2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="CD2" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="CE2" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="CF2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="CG2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="CH2" t="s">
         <v>132</v>
       </c>
       <c r="CI2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="CJ2" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="CK2" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="CL2" t="s">
         <v>123</v>
@@ -1926,250 +1994,268 @@
         <v>123</v>
       </c>
       <c r="CN2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>146</v>
+      </c>
+      <c r="CP2" t="s">
+        <v>147</v>
+      </c>
+      <c r="CQ2" t="s">
         <v>123</v>
       </c>
-      <c r="CO2" t="s">
+      <c r="CR2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CS2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CT2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CU2" t="s">
         <v>132</v>
       </c>
-      <c r="CP2" t="s">
+      <c r="CV2" t="s">
         <v>148</v>
       </c>
-      <c r="CQ2" t="s">
+      <c r="CW2" t="s">
         <v>132</v>
       </c>
-      <c r="CR2" t="s">
+      <c r="CX2" t="s">
         <v>149</v>
       </c>
-      <c r="CS2" t="s">
+      <c r="CY2" t="s">
         <v>149</v>
       </c>
-      <c r="CT2" t="s">
+      <c r="CZ2" t="s">
         <v>150</v>
       </c>
-      <c r="CU2" t="s">
+      <c r="DA2" t="s">
         <v>151</v>
       </c>
-      <c r="CV2" t="s">
+      <c r="DB2" t="s">
         <v>132</v>
       </c>
-      <c r="CW2" t="s">
+      <c r="DC2" t="s">
         <v>152</v>
       </c>
-      <c r="CX2" t="s">
+      <c r="DD2" t="s">
         <v>153</v>
       </c>
-      <c r="CY2" t="s">
+      <c r="DE2" t="s">
         <v>132</v>
       </c>
-      <c r="CZ2" t="s">
+      <c r="DF2" t="s">
         <v>154</v>
       </c>
-      <c r="DA2" t="s">
+      <c r="DG2" t="s">
         <v>155</v>
       </c>
-      <c r="DB2" t="s">
+      <c r="DH2" t="s">
         <v>156</v>
       </c>
-      <c r="DC2" t="s">
+      <c r="DI2" t="s">
         <v>132</v>
       </c>
-      <c r="DD2" t="s">
+      <c r="DJ2" t="s">
         <v>157</v>
       </c>
-      <c r="DE2" t="s">
+      <c r="DK2" t="s">
         <v>149</v>
       </c>
-      <c r="DF2" t="s">
+      <c r="DL2" t="s">
         <v>148</v>
       </c>
-      <c r="DG2" t="s">
+      <c r="DM2" t="s">
         <v>158</v>
-      </c>
-      <c r="DH2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DI2" t="s">
-        <v>158</v>
-      </c>
-      <c r="DJ2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DK2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DL2" t="s">
-        <v>126</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>160</v>
       </c>
       <c r="DN2" t="s">
         <v>132</v>
       </c>
       <c r="DO2" t="s">
+        <v>158</v>
+      </c>
+      <c r="DP2" t="s">
+        <v>159</v>
+      </c>
+      <c r="DQ2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DR2" t="s">
+        <v>126</v>
+      </c>
+      <c r="DS2" t="s">
+        <v>160</v>
+      </c>
+      <c r="DT2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DU2" t="s">
         <v>161</v>
       </c>
-      <c r="DP2" t="s">
+      <c r="DV2" t="s">
         <v>162</v>
       </c>
-      <c r="DQ2" t="s">
+      <c r="DW2" t="s">
         <v>129</v>
       </c>
-      <c r="DR2" t="s">
+      <c r="DX2" t="s">
         <v>132</v>
       </c>
-      <c r="DS2" t="s">
+      <c r="DY2" t="s">
         <v>163</v>
       </c>
-      <c r="DT2" t="s">
+      <c r="DZ2" t="s">
         <v>164</v>
       </c>
-      <c r="DU2" t="s">
+      <c r="EA2" t="s">
         <v>165</v>
       </c>
-      <c r="DV2" t="s">
+      <c r="EB2" t="s">
         <v>166</v>
       </c>
-      <c r="DW2" t="s">
+      <c r="EC2" t="s">
         <v>167</v>
       </c>
-      <c r="DX2" t="s">
+      <c r="ED2" t="s">
         <v>168</v>
       </c>
-      <c r="DY2" t="s">
+      <c r="EE2" t="s">
         <v>169</v>
       </c>
-      <c r="DZ2" t="s">
+      <c r="EF2" t="s">
         <v>126</v>
       </c>
-      <c r="EA2" t="s">
+      <c r="EG2" t="s">
         <v>170</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="43">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 CK2:CN2 AF2 AI2:AM2 AT2 AX2 AZ2 BB2 BD2 CD2 CF2:CG2 K2:X2 Z2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 CQ2:CT2 AL2 AO2:AS2 AZ2 BD2 BF2 BH2 BJ2 CJ2 CL2:CM2 K2:X2 Z2 AE2:AF2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2 BM2 DV2 DY2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2 BN2 BQ2 BT2 BV2 CB2 CE2 CH2 CO2 CQ2 CV2 CY2 DC2 DH2 DK2 DN2 DR2" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2 BS2 EB2 EE2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2 BT2 BW2 BZ2 CB2 CH2 CK2 CN2 CU2 CW2 DB2 DE2 DI2 DN2 DQ2 DT2 DX2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J2 CI2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J2 CO2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DB2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DL2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DR2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DO2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DP2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DV2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DW2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DW2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Berdiri,Telentang"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AD2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AW2 AY2 BA2 BC2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2:BC2 BE2 BG2 BI2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2" xr:uid="{A76BCFDA-99B4-BC4C-9EB2-288C4CC41003}">

</xml_diff>

<commit_message>
telinga mata anak done and wip hepatitis B
</commit_message>
<xml_diff>
--- a/dataset/remaja.xlsx
+++ b/dataset/remaja.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161121ED-0670-BD4F-A8AF-B74F5709EE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CA3AB2-A705-B948-A032-3D45F1EF5DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,7 +141,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="BE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -156,7 +156,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="CB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -171,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="CG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -186,7 +186,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="CJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -201,7 +201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="DA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -216,7 +216,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="DS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -236,7 +236,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="198">
   <si>
     <t>batas_awal</t>
   </si>
@@ -794,6 +794,42 @@
   </si>
   <si>
     <t>gds</t>
+  </si>
+  <si>
+    <t>gangguan_pendengaran_kanan</t>
+  </si>
+  <si>
+    <t>gangguan_pendengaran_kiri</t>
+  </si>
+  <si>
+    <t>serumen_impaksi_kanan</t>
+  </si>
+  <si>
+    <t>serumen_impaksi_kiri</t>
+  </si>
+  <si>
+    <t>infeksi_telinga_kanan</t>
+  </si>
+  <si>
+    <t>infeksi_telinga_kiri</t>
+  </si>
+  <si>
+    <t>selaput_mata_merah_kanan</t>
+  </si>
+  <si>
+    <t>selaput_mata_merah_kiri</t>
+  </si>
+  <si>
+    <t>tajam_penglihatan_kanan</t>
+  </si>
+  <si>
+    <t>Normal (visus 6/6 - 6/9)</t>
+  </si>
+  <si>
+    <t>tajam_penglihatan_kiri</t>
+  </si>
+  <si>
+    <t>menggunakan_kacamata</t>
   </si>
 </sst>
 </file>
@@ -1223,7 +1259,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EG2"/>
+  <dimension ref="A1:ER2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1240,92 +1276,101 @@
     <col min="18" max="20" width="9" bestFit="1" customWidth="1"/>
     <col min="21" max="24" width="13" bestFit="1" customWidth="1"/>
     <col min="25" max="26" width="13" customWidth="1"/>
-    <col min="27" max="34" width="14.33203125" customWidth="1"/>
-    <col min="35" max="35" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="19" bestFit="1" customWidth="1"/>
-    <col min="37" max="39" width="19" customWidth="1"/>
-    <col min="40" max="40" width="25" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="14.83203125" customWidth="1"/>
-    <col min="47" max="47" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="10" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="16" bestFit="1" customWidth="1"/>
-    <col min="51" max="52" width="13.6640625" customWidth="1"/>
-    <col min="53" max="53" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="54" max="55" width="13.6640625" customWidth="1"/>
-    <col min="56" max="56" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="57" max="61" width="22.5" customWidth="1"/>
-    <col min="62" max="62" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="63" max="66" width="22.5" customWidth="1"/>
-    <col min="67" max="67" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="22.83203125" customWidth="1"/>
-    <col min="72" max="72" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="16.1640625" customWidth="1"/>
-    <col min="74" max="74" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="76" max="77" width="12.33203125" customWidth="1"/>
-    <col min="78" max="78" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="14.1640625" customWidth="1"/>
-    <col min="80" max="80" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="23.6640625" customWidth="1"/>
-    <col min="83" max="83" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="12.83203125" customWidth="1"/>
-    <col min="89" max="89" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="17.5" customWidth="1"/>
-    <col min="92" max="92" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="13" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="96" max="98" width="19.5" customWidth="1"/>
-    <col min="99" max="99" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="9.83203125" customWidth="1"/>
-    <col min="101" max="101" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="102" max="105" width="11.5" customWidth="1"/>
-    <col min="106" max="106" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="9" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="18.1640625" customWidth="1"/>
-    <col min="113" max="113" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="115" max="117" width="8.33203125" customWidth="1"/>
-    <col min="118" max="118" width="22" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="14" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="14" customWidth="1"/>
-    <col min="123" max="123" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="27" max="30" width="14.33203125" customWidth="1"/>
+    <col min="31" max="31" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="37" width="24.1640625" customWidth="1"/>
+    <col min="38" max="38" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="39" max="44" width="24.1640625" customWidth="1"/>
+    <col min="45" max="45" width="14.33203125" customWidth="1"/>
+    <col min="46" max="46" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="19" bestFit="1" customWidth="1"/>
+    <col min="48" max="50" width="19" customWidth="1"/>
+    <col min="51" max="51" width="25" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="14.83203125" customWidth="1"/>
+    <col min="58" max="58" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="10" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="16" bestFit="1" customWidth="1"/>
+    <col min="62" max="63" width="13.6640625" customWidth="1"/>
+    <col min="64" max="64" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="65" max="66" width="13.6640625" customWidth="1"/>
+    <col min="67" max="67" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="68" max="72" width="22.5" customWidth="1"/>
+    <col min="73" max="73" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="74" max="77" width="22.5" customWidth="1"/>
+    <col min="78" max="78" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="22.83203125" customWidth="1"/>
+    <col min="83" max="83" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="16.1640625" customWidth="1"/>
+    <col min="85" max="85" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="87" max="88" width="12.33203125" customWidth="1"/>
+    <col min="89" max="89" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="14.1640625" customWidth="1"/>
+    <col min="91" max="91" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="23.6640625" customWidth="1"/>
+    <col min="94" max="94" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="12.83203125" customWidth="1"/>
+    <col min="100" max="100" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="17.5" customWidth="1"/>
+    <col min="103" max="103" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="13" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="107" max="109" width="19.5" customWidth="1"/>
+    <col min="110" max="110" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="9.83203125" customWidth="1"/>
+    <col min="112" max="112" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="113" max="116" width="11.5" customWidth="1"/>
+    <col min="117" max="117" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="9" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="18.1640625" customWidth="1"/>
     <col min="124" max="124" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="18.1640625" customWidth="1"/>
-    <col min="126" max="126" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="129" max="131" width="18.1640625" customWidth="1"/>
-    <col min="132" max="132" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="133" max="133" width="35" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="18.1640625" customWidth="1"/>
-    <col min="136" max="136" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="137" max="137" width="10.83203125" customWidth="1"/>
+    <col min="125" max="125" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="126" max="128" width="8.33203125" customWidth="1"/>
+    <col min="129" max="129" width="22" bestFit="1" customWidth="1"/>
+    <col min="130" max="130" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="132" max="132" width="14" bestFit="1" customWidth="1"/>
+    <col min="133" max="133" width="14" customWidth="1"/>
+    <col min="134" max="134" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="135" max="135" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="136" max="136" width="18.1640625" customWidth="1"/>
+    <col min="137" max="137" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="138" max="138" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="139" max="139" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="140" max="142" width="18.1640625" customWidth="1"/>
+    <col min="143" max="143" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="144" max="144" width="35" bestFit="1" customWidth="1"/>
+    <col min="145" max="145" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="146" max="146" width="18.1640625" customWidth="1"/>
+    <col min="147" max="147" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="148" max="148" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:137" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:148" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1423,318 +1468,351 @@
       <c r="AG1" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="AH1" s="2"/>
-      <c r="AI1" t="s">
+      <c r="AH1" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="AL1" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AO1" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="AP1" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="AQ1" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="AS1" s="2"/>
+      <c r="AT1" t="s">
         <v>16</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AU1" t="s">
         <v>17</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AV1" t="s">
         <v>18</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AW1" t="s">
         <v>19</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AX1" t="s">
         <v>20</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AY1" t="s">
         <v>21</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AZ1" t="s">
         <v>22</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="BA1" t="s">
         <v>23</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="BB1" t="s">
         <v>24</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="BC1" t="s">
         <v>25</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="BD1" t="s">
         <v>26</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="BE1" t="s">
         <v>27</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="BF1" t="s">
         <v>28</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BG1" t="s">
         <v>29</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BH1" t="s">
         <v>30</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BI1" t="s">
         <v>31</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BJ1" t="s">
         <v>32</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BK1" t="s">
         <v>33</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BL1" t="s">
         <v>34</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BM1" t="s">
         <v>35</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BN1" t="s">
         <v>36</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BO1" t="s">
         <v>37</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BP1" t="s">
         <v>38</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BQ1" t="s">
         <v>39</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BR1" t="s">
         <v>40</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BS1" t="s">
         <v>41</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BT1" t="s">
         <v>42</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BU1" t="s">
         <v>43</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BV1" t="s">
         <v>44</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BW1" t="s">
         <v>45</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BX1" t="s">
         <v>46</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BY1" t="s">
         <v>47</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BZ1" t="s">
         <v>48</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="CA1" t="s">
         <v>49</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="CB1" t="s">
         <v>50</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="CC1" t="s">
         <v>51</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="CD1" t="s">
         <v>52</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="CE1" t="s">
         <v>53</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CF1" t="s">
         <v>54</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CG1" t="s">
         <v>55</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CH1" t="s">
         <v>56</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CI1" t="s">
         <v>57</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CJ1" t="s">
         <v>58</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CK1" t="s">
         <v>59</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CL1" t="s">
         <v>60</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CM1" t="s">
         <v>61</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CN1" t="s">
         <v>62</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CO1" t="s">
         <v>63</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CP1" t="s">
         <v>64</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CQ1" t="s">
         <v>65</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CR1" t="s">
         <v>66</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CS1" t="s">
         <v>67</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CT1" t="s">
         <v>68</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CU1" t="s">
         <v>69</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CV1" t="s">
         <v>70</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CW1" t="s">
         <v>71</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CX1" t="s">
         <v>72</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CY1" t="s">
         <v>73</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CZ1" t="s">
         <v>74</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="DA1" t="s">
         <v>75</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="DB1" t="s">
         <v>76</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="DC1" t="s">
         <v>77</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="DD1" t="s">
         <v>78</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="DE1" t="s">
         <v>79</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="DF1" t="s">
         <v>80</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="DG1" t="s">
         <v>81</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="DH1" t="s">
         <v>82</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="DI1" t="s">
         <v>83</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="DJ1" t="s">
         <v>84</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DK1" t="s">
         <v>85</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DL1" t="s">
         <v>86</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DM1" t="s">
         <v>87</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DN1" t="s">
         <v>88</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DO1" t="s">
         <v>89</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DP1" t="s">
         <v>90</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DQ1" t="s">
         <v>91</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DR1" t="s">
         <v>92</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DS1" t="s">
         <v>93</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DT1" t="s">
         <v>94</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DU1" t="s">
         <v>95</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DV1" t="s">
         <v>96</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DW1" t="s">
         <v>97</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DX1" t="s">
         <v>98</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DY1" t="s">
         <v>99</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DZ1" t="s">
         <v>100</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="EA1" t="s">
         <v>101</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="EB1" t="s">
         <v>102</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="EC1" t="s">
         <v>103</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="ED1" t="s">
         <v>104</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="EE1" t="s">
         <v>105</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="EF1" t="s">
         <v>106</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="EG1" t="s">
         <v>107</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="EH1" t="s">
         <v>108</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="EI1" t="s">
         <v>109</v>
       </c>
-      <c r="DY1" t="s">
+      <c r="EJ1" t="s">
         <v>110</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="EK1" t="s">
         <v>111</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="EL1" t="s">
         <v>112</v>
       </c>
-      <c r="EB1" t="s">
+      <c r="EM1" t="s">
         <v>113</v>
       </c>
-      <c r="EC1" t="s">
+      <c r="EN1" t="s">
         <v>114</v>
       </c>
-      <c r="ED1" t="s">
+      <c r="EO1" t="s">
         <v>115</v>
       </c>
-      <c r="EE1" t="s">
+      <c r="EP1" t="s">
         <v>116</v>
       </c>
-      <c r="EF1" t="s">
+      <c r="EQ1" t="s">
         <v>117</v>
       </c>
-      <c r="EG1" t="s">
+      <c r="ER1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:137" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:148" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>119</v>
       </c>
@@ -1822,440 +1900,473 @@
       <c r="AG2">
         <v>120</v>
       </c>
+      <c r="AH2" t="s">
+        <v>126</v>
+      </c>
       <c r="AI2" t="s">
+        <v>126</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>142</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>142</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>143</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>143</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>126</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>126</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>195</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>195</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>122</v>
+      </c>
+      <c r="AT2" t="s">
         <v>125</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AU2" t="s">
         <v>126</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AV2" t="s">
         <v>127</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AW2" t="s">
         <v>123</v>
       </c>
-      <c r="AM2">
+      <c r="AX2">
         <v>10</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AY2" t="s">
         <v>128</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>126</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>124</v>
-      </c>
-      <c r="AV2">
-        <v>2900</v>
-      </c>
-      <c r="AW2">
-        <v>6000</v>
-      </c>
-      <c r="AX2">
-        <v>80</v>
-      </c>
-      <c r="AY2">
-        <v>90</v>
       </c>
       <c r="AZ2" t="s">
         <v>123</v>
       </c>
       <c r="BA2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="BB2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="BC2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="BD2" t="s">
         <v>123</v>
       </c>
       <c r="BE2" t="s">
+        <v>126</v>
+      </c>
+      <c r="BF2" t="s">
+        <v>124</v>
+      </c>
+      <c r="BG2">
+        <v>2900</v>
+      </c>
+      <c r="BH2">
+        <v>6000</v>
+      </c>
+      <c r="BI2">
+        <v>80</v>
+      </c>
+      <c r="BJ2">
+        <v>90</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>123</v>
+      </c>
+      <c r="BL2" t="s">
         <v>129</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BM2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BO2" t="s">
         <v>123</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BP2" t="s">
         <v>129</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BQ2" t="s">
         <v>123</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BR2" t="s">
         <v>129</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BS2" t="s">
+        <v>123</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>129</v>
+      </c>
+      <c r="BU2" t="s">
         <v>122</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BV2" t="s">
         <v>130</v>
       </c>
-      <c r="BL2">
+      <c r="BW2">
         <v>30122025</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BX2" t="s">
         <v>126</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BY2" t="s">
         <v>131</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>132</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>133</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>134</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>135</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>136</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>132</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>137</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>138</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>132</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>139</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>140</v>
       </c>
       <c r="BZ2" t="s">
         <v>132</v>
       </c>
       <c r="CA2" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="CB2" t="s">
+        <v>134</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>135</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>136</v>
+      </c>
+      <c r="CE2" t="s">
         <v>132</v>
       </c>
-      <c r="CC2" t="s">
-        <v>142</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>143</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>144</v>
-      </c>
       <c r="CF2" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="CG2" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="CH2" t="s">
         <v>132</v>
       </c>
       <c r="CI2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="CJ2" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="CK2" t="s">
         <v>132</v>
       </c>
       <c r="CL2" t="s">
+        <v>141</v>
+      </c>
+      <c r="CM2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CN2" t="s">
+        <v>142</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>143</v>
+      </c>
+      <c r="CP2" t="s">
+        <v>144</v>
+      </c>
+      <c r="CQ2" t="s">
+        <v>126</v>
+      </c>
+      <c r="CR2" t="s">
+        <v>126</v>
+      </c>
+      <c r="CS2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CT2" t="s">
+        <v>145</v>
+      </c>
+      <c r="CU2" t="s">
+        <v>122</v>
+      </c>
+      <c r="CV2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CW2" t="s">
         <v>123</v>
       </c>
-      <c r="CM2" t="s">
+      <c r="CX2" t="s">
         <v>123</v>
       </c>
-      <c r="CN2" t="s">
+      <c r="CY2" t="s">
         <v>132</v>
       </c>
-      <c r="CO2" t="s">
+      <c r="CZ2" t="s">
         <v>146</v>
       </c>
-      <c r="CP2" t="s">
+      <c r="DA2" t="s">
         <v>147</v>
       </c>
-      <c r="CQ2" t="s">
+      <c r="DB2" t="s">
         <v>123</v>
       </c>
-      <c r="CR2" t="s">
+      <c r="DC2" t="s">
         <v>123</v>
       </c>
-      <c r="CS2" t="s">
+      <c r="DD2" t="s">
         <v>123</v>
       </c>
-      <c r="CT2" t="s">
+      <c r="DE2" t="s">
         <v>123</v>
       </c>
-      <c r="CU2" t="s">
+      <c r="DF2" t="s">
         <v>132</v>
       </c>
-      <c r="CV2" t="s">
+      <c r="DG2" t="s">
         <v>148</v>
       </c>
-      <c r="CW2" t="s">
+      <c r="DH2" t="s">
         <v>132</v>
       </c>
-      <c r="CX2" t="s">
+      <c r="DI2" t="s">
         <v>149</v>
       </c>
-      <c r="CY2" t="s">
+      <c r="DJ2" t="s">
         <v>149</v>
       </c>
-      <c r="CZ2" t="s">
+      <c r="DK2" t="s">
         <v>150</v>
       </c>
-      <c r="DA2" t="s">
+      <c r="DL2" t="s">
         <v>151</v>
       </c>
-      <c r="DB2" t="s">
+      <c r="DM2" t="s">
         <v>132</v>
       </c>
-      <c r="DC2" t="s">
+      <c r="DN2" t="s">
         <v>152</v>
       </c>
-      <c r="DD2" t="s">
+      <c r="DO2" t="s">
         <v>153</v>
       </c>
-      <c r="DE2" t="s">
+      <c r="DP2" t="s">
         <v>132</v>
       </c>
-      <c r="DF2" t="s">
+      <c r="DQ2" t="s">
         <v>154</v>
       </c>
-      <c r="DG2" t="s">
+      <c r="DR2" t="s">
         <v>155</v>
       </c>
-      <c r="DH2" t="s">
+      <c r="DS2" t="s">
         <v>156</v>
-      </c>
-      <c r="DI2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DJ2" t="s">
-        <v>157</v>
-      </c>
-      <c r="DK2" t="s">
-        <v>149</v>
-      </c>
-      <c r="DL2" t="s">
-        <v>148</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>158</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DO2" t="s">
-        <v>158</v>
-      </c>
-      <c r="DP2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DQ2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>126</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>160</v>
       </c>
       <c r="DT2" t="s">
         <v>132</v>
       </c>
       <c r="DU2" t="s">
+        <v>157</v>
+      </c>
+      <c r="DV2" t="s">
+        <v>149</v>
+      </c>
+      <c r="DW2" t="s">
+        <v>148</v>
+      </c>
+      <c r="DX2" t="s">
+        <v>158</v>
+      </c>
+      <c r="DY2" t="s">
+        <v>132</v>
+      </c>
+      <c r="DZ2" t="s">
+        <v>158</v>
+      </c>
+      <c r="EA2" t="s">
+        <v>159</v>
+      </c>
+      <c r="EB2" t="s">
+        <v>132</v>
+      </c>
+      <c r="EC2" t="s">
+        <v>126</v>
+      </c>
+      <c r="ED2" t="s">
+        <v>160</v>
+      </c>
+      <c r="EE2" t="s">
+        <v>132</v>
+      </c>
+      <c r="EF2" t="s">
         <v>161</v>
       </c>
-      <c r="DV2" t="s">
+      <c r="EG2" t="s">
         <v>162</v>
       </c>
-      <c r="DW2" t="s">
+      <c r="EH2" t="s">
         <v>129</v>
       </c>
-      <c r="DX2" t="s">
+      <c r="EI2" t="s">
         <v>132</v>
       </c>
-      <c r="DY2" t="s">
+      <c r="EJ2" t="s">
         <v>163</v>
       </c>
-      <c r="DZ2" t="s">
+      <c r="EK2" t="s">
         <v>164</v>
       </c>
-      <c r="EA2" t="s">
+      <c r="EL2" t="s">
         <v>165</v>
       </c>
-      <c r="EB2" t="s">
+      <c r="EM2" t="s">
         <v>166</v>
       </c>
-      <c r="EC2" t="s">
+      <c r="EN2" t="s">
         <v>167</v>
       </c>
-      <c r="ED2" t="s">
+      <c r="EO2" t="s">
         <v>168</v>
       </c>
-      <c r="EE2" t="s">
+      <c r="EP2" t="s">
         <v>169</v>
       </c>
-      <c r="EF2" t="s">
+      <c r="EQ2" t="s">
         <v>126</v>
       </c>
-      <c r="EG2" t="s">
+      <c r="ER2" t="s">
         <v>170</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="43">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 CQ2:CT2 AL2 AO2:AS2 AZ2 BD2 BF2 BH2 BJ2 CJ2 CL2:CM2 K2:X2 Z2 AE2:AF2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="45">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 DB2:DE2 AW2 AZ2:BD2 BK2 BO2 BQ2 BS2 BU2 CU2 CW2:CX2 K2:X2 Z2 AE2:AF2 AR2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2 BS2 EB2 EE2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2 BT2 BW2 BZ2 CB2 CH2 CK2 CN2 CU2 CW2 DB2 DE2 DI2 DN2 DQ2 DT2 DX2" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AY2 CD2 EM2 EP2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2 CE2 CH2 CK2 CM2 CS2 CV2 CY2 DF2 DH2 DM2 DP2 DT2 DY2 EB2 EE2 EI2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2 AJ2:AK2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2 AL2:AM2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2 AN2:AO2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J2 CO2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J2 CZ2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DR2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DR2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DV2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EG2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DW2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EH2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EJ2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EK2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EN2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Berdiri,Telentang"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2:BC2 BE2 BG2 BI2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BN2 BP2 BR2 BT2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2" xr:uid="{A76BCFDA-99B4-BC4C-9EB2-288C4CC41003}">
@@ -2268,6 +2379,12 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2:AI2" xr:uid="{D8788161-8880-9442-A20F-C2CE2C1A3CD0}">
+      <formula1>"Normal,Ada indikasi gangguan pendengaran"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2:AQ2" xr:uid="{D2187A34-3D8D-2F49-BAA8-8ABAFEDA0518}">
+      <formula1>"Normal (visus 6/6 - 6/9),Ada indikasi gangguan penglihatan (visus &lt;6/9)"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
telinga wip hepatitis B
</commit_message>
<xml_diff>
--- a/dataset/remaja.xlsx
+++ b/dataset/remaja.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CA3AB2-A705-B948-A032-3D45F1EF5DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59774B37-0557-0042-AD91-A9473D783EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,7 +141,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -156,7 +156,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="BI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -171,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="BN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -186,7 +186,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="BQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -201,7 +201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="CH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -216,7 +216,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="CZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -236,7 +236,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="174">
   <si>
     <t>batas_awal</t>
   </si>
@@ -286,21 +286,6 @@
     <t>tinggi_badan</t>
   </si>
   <si>
-    <t>posisi_pengukuran</t>
-  </si>
-  <si>
-    <t>status_lingkar_kepala</t>
-  </si>
-  <si>
-    <t>hasil_kpsp</t>
-  </si>
-  <si>
-    <t>m_chat_1</t>
-  </si>
-  <si>
-    <t>m_chat_2</t>
-  </si>
-  <si>
     <t>pernah_batuk_tidak_sembuh</t>
   </si>
   <si>
@@ -337,51 +322,6 @@
     <t>pjb_kaki</t>
   </si>
   <si>
-    <t>darah_tumit</t>
-  </si>
-  <si>
-    <t>shk</t>
-  </si>
-  <si>
-    <t>g6pd</t>
-  </si>
-  <si>
-    <t>hak</t>
-  </si>
-  <si>
-    <t>dilakukan_konfirmasi_shk</t>
-  </si>
-  <si>
-    <t>hasil_konfirm_shk</t>
-  </si>
-  <si>
-    <t>dilakukan_konfirmasi_g6pd</t>
-  </si>
-  <si>
-    <t>hasil_konfirm_g6pd</t>
-  </si>
-  <si>
-    <t>dilakukan_konfirmasi_hak</t>
-  </si>
-  <si>
-    <t>hasil_konfirm_hak</t>
-  </si>
-  <si>
-    <t>dilakukan_edukasi_warna_kulit_dan_tinja</t>
-  </si>
-  <si>
-    <t>nilai_hasil_kramer</t>
-  </si>
-  <si>
-    <t>tgl_pemeriksaan_kramer</t>
-  </si>
-  <si>
-    <t>kramer_bayi_kuning</t>
-  </si>
-  <si>
-    <t>derajat_warna_tinja</t>
-  </si>
-  <si>
     <t>periksa_tbc</t>
   </si>
   <si>
@@ -613,25 +553,13 @@
     <t>Sudah</t>
   </si>
   <si>
-    <t>Berdiri</t>
-  </si>
-  <si>
     <t>Normal</t>
   </si>
   <si>
-    <t>Perkembangan sesuai usia</t>
-  </si>
-  <si>
     <t>Tidak batuk</t>
   </si>
   <si>
     <t>Negatif</t>
-  </si>
-  <si>
-    <t>Bayi Kuning Kramer 1-3</t>
-  </si>
-  <si>
-    <t>&gt;3 Normal</t>
   </si>
   <si>
     <t>True</t>
@@ -1259,7 +1187,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:ER2"/>
+  <dimension ref="A1:DY2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1286,91 +1214,82 @@
     <col min="38" max="38" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="39" max="44" width="24.1640625" customWidth="1"/>
     <col min="45" max="45" width="14.33203125" customWidth="1"/>
-    <col min="46" max="46" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="19" bestFit="1" customWidth="1"/>
-    <col min="48" max="50" width="19" customWidth="1"/>
-    <col min="51" max="51" width="25" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="14.83203125" customWidth="1"/>
-    <col min="58" max="58" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="10" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="16" bestFit="1" customWidth="1"/>
-    <col min="62" max="63" width="13.6640625" customWidth="1"/>
-    <col min="64" max="64" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="65" max="66" width="13.6640625" customWidth="1"/>
-    <col min="67" max="67" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="68" max="72" width="22.5" customWidth="1"/>
-    <col min="73" max="73" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="74" max="77" width="22.5" customWidth="1"/>
-    <col min="78" max="78" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="22.83203125" customWidth="1"/>
-    <col min="83" max="83" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="16.1640625" customWidth="1"/>
-    <col min="85" max="85" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="88" width="12.33203125" customWidth="1"/>
-    <col min="89" max="89" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="14.1640625" customWidth="1"/>
-    <col min="91" max="91" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="23.6640625" customWidth="1"/>
-    <col min="94" max="94" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="12.83203125" customWidth="1"/>
-    <col min="100" max="100" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="17.5" customWidth="1"/>
-    <col min="103" max="103" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="13" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="107" max="109" width="19.5" customWidth="1"/>
-    <col min="110" max="110" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="9.83203125" customWidth="1"/>
-    <col min="112" max="112" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="113" max="116" width="11.5" customWidth="1"/>
-    <col min="117" max="117" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="9" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="18.1640625" customWidth="1"/>
-    <col min="124" max="124" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="126" max="128" width="8.33203125" customWidth="1"/>
-    <col min="129" max="129" width="22" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="14" bestFit="1" customWidth="1"/>
-    <col min="133" max="133" width="14" customWidth="1"/>
-    <col min="134" max="134" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="136" max="136" width="18.1640625" customWidth="1"/>
-    <col min="137" max="137" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="138" max="138" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="139" max="139" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="140" max="142" width="18.1640625" customWidth="1"/>
-    <col min="143" max="143" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="144" max="144" width="35" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="146" max="146" width="18.1640625" customWidth="1"/>
-    <col min="147" max="147" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="148" max="148" width="10.83203125" customWidth="1"/>
+    <col min="46" max="46" width="25" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="14.83203125" customWidth="1"/>
+    <col min="54" max="54" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="10" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="16" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="13.6640625" customWidth="1"/>
+    <col min="59" max="59" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="22.83203125" customWidth="1"/>
+    <col min="64" max="64" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="16.1640625" customWidth="1"/>
+    <col min="66" max="66" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="68" max="69" width="12.33203125" customWidth="1"/>
+    <col min="70" max="70" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="14.1640625" customWidth="1"/>
+    <col min="72" max="72" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="23.6640625" customWidth="1"/>
+    <col min="75" max="75" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="12.83203125" customWidth="1"/>
+    <col min="81" max="81" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="17.5" customWidth="1"/>
+    <col min="84" max="84" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="13" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="88" max="90" width="19.5" customWidth="1"/>
+    <col min="91" max="91" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="9.83203125" customWidth="1"/>
+    <col min="93" max="93" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="94" max="97" width="11.5" customWidth="1"/>
+    <col min="98" max="98" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="9" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="18.1640625" customWidth="1"/>
+    <col min="105" max="105" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="107" max="109" width="8.33203125" customWidth="1"/>
+    <col min="110" max="110" width="22" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="14" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="14" customWidth="1"/>
+    <col min="115" max="115" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="18.1640625" customWidth="1"/>
+    <col min="118" max="118" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="121" max="123" width="18.1640625" customWidth="1"/>
+    <col min="124" max="124" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="35" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="18.1640625" customWidth="1"/>
+    <col min="128" max="128" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:148" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:129" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1414,37 +1333,37 @@
         <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>173</v>
+        <v>149</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>176</v>
+        <v>152</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>177</v>
+        <v>153</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>178</v>
+        <v>154</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>179</v>
+        <v>155</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>181</v>
+        <v>157</v>
       </c>
       <c r="Z1" s="2"/>
       <c r="AA1" t="s">
@@ -1454,52 +1373,52 @@
         <v>15</v>
       </c>
       <c r="AC1" s="2" t="s">
-        <v>182</v>
+        <v>158</v>
       </c>
       <c r="AD1" s="2" t="s">
-        <v>183</v>
+        <v>159</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="AF1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="AJ1" s="2" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="AK1" s="2" t="s">
-        <v>189</v>
+        <v>165</v>
       </c>
       <c r="AL1" s="2" t="s">
-        <v>190</v>
+        <v>166</v>
       </c>
       <c r="AM1" s="2" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
       <c r="AN1" s="2" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="AO1" s="2" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
       <c r="AP1" s="2" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="AQ1" s="2" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="AR1" s="2" t="s">
-        <v>197</v>
+        <v>173</v>
       </c>
       <c r="AS1" s="2"/>
       <c r="AT1" t="s">
@@ -1523,364 +1442,304 @@
       <c r="AZ1" t="s">
         <v>22</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>23</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>24</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>25</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>26</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>27</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>28</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>29</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>30</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>31</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BK1" t="s">
         <v>32</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>33</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" t="s">
         <v>34</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>35</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>36</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BP1" t="s">
         <v>37</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>38</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>39</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>40</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BT1" t="s">
         <v>41</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BU1" t="s">
         <v>42</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BV1" t="s">
         <v>43</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BW1" t="s">
         <v>44</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BX1" t="s">
         <v>45</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BY1" t="s">
         <v>46</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BZ1" t="s">
         <v>47</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CA1" t="s">
         <v>48</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CB1" t="s">
         <v>49</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CC1" t="s">
         <v>50</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CD1" t="s">
         <v>51</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CE1" t="s">
         <v>52</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CF1" t="s">
         <v>53</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CG1" t="s">
         <v>54</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CH1" t="s">
         <v>55</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CI1" t="s">
         <v>56</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CJ1" t="s">
         <v>57</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CK1" t="s">
         <v>58</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CL1" t="s">
         <v>59</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CM1" t="s">
         <v>60</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CN1" t="s">
         <v>61</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CO1" t="s">
         <v>62</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CP1" t="s">
         <v>63</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CQ1" t="s">
         <v>64</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CR1" t="s">
         <v>65</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CS1" t="s">
         <v>66</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CT1" t="s">
         <v>67</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CU1" t="s">
         <v>68</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CV1" t="s">
         <v>69</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="CW1" t="s">
         <v>70</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="CX1" t="s">
         <v>71</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="CY1" t="s">
         <v>72</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="CZ1" t="s">
         <v>73</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DA1" t="s">
         <v>74</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DB1" t="s">
         <v>75</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DC1" t="s">
         <v>76</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DD1" t="s">
         <v>77</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DE1" t="s">
         <v>78</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DF1" t="s">
         <v>79</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DG1" t="s">
         <v>80</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DH1" t="s">
         <v>81</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DI1" t="s">
         <v>82</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DJ1" t="s">
         <v>83</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DK1" t="s">
         <v>84</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DL1" t="s">
         <v>85</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DM1" t="s">
         <v>86</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DN1" t="s">
         <v>87</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DO1" t="s">
         <v>88</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DP1" t="s">
         <v>89</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="DQ1" t="s">
         <v>90</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="DR1" t="s">
         <v>91</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="DS1" t="s">
         <v>92</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="DT1" t="s">
         <v>93</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="DU1" t="s">
         <v>94</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="DV1" t="s">
         <v>95</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="DW1" t="s">
         <v>96</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="DX1" t="s">
         <v>97</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="DY1" t="s">
         <v>98</v>
       </c>
-      <c r="DY1" t="s">
+    </row>
+    <row r="2" spans="1:129" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="B2" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="C2" t="s">
         <v>101</v>
       </c>
-      <c r="EB1" t="s">
+      <c r="E2" t="s">
         <v>102</v>
       </c>
-      <c r="EC1" t="s">
-        <v>103</v>
-      </c>
-      <c r="ED1" t="s">
-        <v>104</v>
-      </c>
-      <c r="EE1" t="s">
-        <v>105</v>
-      </c>
-      <c r="EF1" t="s">
+      <c r="G2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H2" t="s">
+        <v>102</v>
+      </c>
+      <c r="I2" t="s">
+        <v>102</v>
+      </c>
+      <c r="J2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" t="s">
+        <v>102</v>
+      </c>
+      <c r="L2" t="s">
+        <v>102</v>
+      </c>
+      <c r="M2" t="s">
+        <v>102</v>
+      </c>
+      <c r="N2" t="s">
+        <v>102</v>
+      </c>
+      <c r="O2" t="s">
+        <v>102</v>
+      </c>
+      <c r="P2" t="s">
+        <v>102</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>102</v>
+      </c>
+      <c r="R2" t="s">
+        <v>102</v>
+      </c>
+      <c r="S2" t="s">
+        <v>102</v>
+      </c>
+      <c r="T2" t="s">
+        <v>102</v>
+      </c>
+      <c r="U2" t="s">
+        <v>102</v>
+      </c>
+      <c r="V2" t="s">
+        <v>102</v>
+      </c>
+      <c r="W2" t="s">
+        <v>102</v>
+      </c>
+      <c r="X2" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y2" t="s">
         <v>106</v>
-      </c>
-      <c r="EG1" t="s">
-        <v>107</v>
-      </c>
-      <c r="EH1" t="s">
-        <v>108</v>
-      </c>
-      <c r="EI1" t="s">
-        <v>109</v>
-      </c>
-      <c r="EJ1" t="s">
-        <v>110</v>
-      </c>
-      <c r="EK1" t="s">
-        <v>111</v>
-      </c>
-      <c r="EL1" t="s">
-        <v>112</v>
-      </c>
-      <c r="EM1" t="s">
-        <v>113</v>
-      </c>
-      <c r="EN1" t="s">
-        <v>114</v>
-      </c>
-      <c r="EO1" t="s">
-        <v>115</v>
-      </c>
-      <c r="EP1" t="s">
-        <v>116</v>
-      </c>
-      <c r="EQ1" t="s">
-        <v>117</v>
-      </c>
-      <c r="ER1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="2" spans="1:148" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E2" t="s">
-        <v>122</v>
-      </c>
-      <c r="G2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H2" t="s">
-        <v>122</v>
-      </c>
-      <c r="I2" t="s">
-        <v>122</v>
-      </c>
-      <c r="J2" t="s">
-        <v>122</v>
-      </c>
-      <c r="K2" t="s">
-        <v>122</v>
-      </c>
-      <c r="L2" t="s">
-        <v>122</v>
-      </c>
-      <c r="M2" t="s">
-        <v>122</v>
-      </c>
-      <c r="N2" t="s">
-        <v>122</v>
-      </c>
-      <c r="O2" t="s">
-        <v>122</v>
-      </c>
-      <c r="P2" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>122</v>
-      </c>
-      <c r="R2" t="s">
-        <v>122</v>
-      </c>
-      <c r="S2" t="s">
-        <v>122</v>
-      </c>
-      <c r="T2" t="s">
-        <v>122</v>
-      </c>
-      <c r="U2" t="s">
-        <v>122</v>
-      </c>
-      <c r="V2" t="s">
-        <v>122</v>
-      </c>
-      <c r="W2" t="s">
-        <v>122</v>
-      </c>
-      <c r="X2" t="s">
-        <v>122</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>128</v>
       </c>
       <c r="AA2">
         <v>50</v>
@@ -1895,479 +1754,398 @@
         <v>80</v>
       </c>
       <c r="AE2" t="s">
-        <v>122</v>
+        <v>102</v>
       </c>
       <c r="AG2">
         <v>120</v>
       </c>
       <c r="AH2" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="AI2" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="AJ2" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="AK2" t="s">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="AL2" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="AM2" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="AN2" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="AO2" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="AP2" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="AQ2" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="AR2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>106</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>105</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>104</v>
+      </c>
+      <c r="BC2">
+        <v>2900</v>
+      </c>
+      <c r="BD2">
+        <v>6000</v>
+      </c>
+      <c r="BE2">
+        <v>80</v>
+      </c>
+      <c r="BF2">
+        <v>90</v>
+      </c>
+      <c r="BG2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>109</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BJ2" t="s">
+        <v>111</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>112</v>
+      </c>
+      <c r="BL2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BM2" t="s">
+        <v>113</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>114</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BP2" t="s">
+        <v>115</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>116</v>
+      </c>
+      <c r="BR2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>117</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>118</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>119</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>120</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>105</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>105</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>121</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>102</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>103</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>103</v>
+      </c>
+      <c r="CF2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CG2" t="s">
         <v>122</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="CH2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CI2" t="s">
+        <v>103</v>
+      </c>
+      <c r="CJ2" t="s">
+        <v>103</v>
+      </c>
+      <c r="CK2" t="s">
+        <v>103</v>
+      </c>
+      <c r="CL2" t="s">
+        <v>103</v>
+      </c>
+      <c r="CM2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CN2" t="s">
+        <v>124</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CP2" t="s">
         <v>125</v>
       </c>
-      <c r="AU2" t="s">
-        <v>126</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>127</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>123</v>
-      </c>
-      <c r="AX2">
-        <v>10</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>128</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>126</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>124</v>
-      </c>
-      <c r="BG2">
-        <v>2900</v>
-      </c>
-      <c r="BH2">
-        <v>6000</v>
-      </c>
-      <c r="BI2">
-        <v>80</v>
-      </c>
-      <c r="BJ2">
-        <v>90</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>129</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>129</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>129</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>129</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>129</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>123</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>129</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>122</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>130</v>
-      </c>
-      <c r="BW2">
-        <v>30122025</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>126</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>131</v>
-      </c>
-      <c r="BZ2" t="s">
-        <v>132</v>
-      </c>
-      <c r="CA2" t="s">
-        <v>133</v>
-      </c>
-      <c r="CB2" t="s">
-        <v>134</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>135</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>136</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>132</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>137</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>138</v>
-      </c>
-      <c r="CH2" t="s">
-        <v>132</v>
-      </c>
-      <c r="CI2" t="s">
-        <v>139</v>
-      </c>
-      <c r="CJ2" t="s">
-        <v>140</v>
-      </c>
-      <c r="CK2" t="s">
-        <v>132</v>
-      </c>
-      <c r="CL2" t="s">
-        <v>141</v>
-      </c>
-      <c r="CM2" t="s">
-        <v>132</v>
-      </c>
-      <c r="CN2" t="s">
-        <v>142</v>
-      </c>
-      <c r="CO2" t="s">
-        <v>143</v>
-      </c>
-      <c r="CP2" t="s">
-        <v>144</v>
-      </c>
       <c r="CQ2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="CR2" t="s">
         <v>126</v>
       </c>
       <c r="CS2" t="s">
+        <v>127</v>
+      </c>
+      <c r="CT2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CU2" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV2" t="s">
+        <v>129</v>
+      </c>
+      <c r="CW2" t="s">
+        <v>108</v>
+      </c>
+      <c r="CX2" t="s">
+        <v>130</v>
+      </c>
+      <c r="CY2" t="s">
+        <v>131</v>
+      </c>
+      <c r="CZ2" t="s">
         <v>132</v>
       </c>
-      <c r="CT2" t="s">
+      <c r="DA2" t="s">
+        <v>108</v>
+      </c>
+      <c r="DB2" t="s">
+        <v>133</v>
+      </c>
+      <c r="DC2" t="s">
+        <v>125</v>
+      </c>
+      <c r="DD2" t="s">
+        <v>124</v>
+      </c>
+      <c r="DE2" t="s">
+        <v>134</v>
+      </c>
+      <c r="DF2" t="s">
+        <v>108</v>
+      </c>
+      <c r="DG2" t="s">
+        <v>134</v>
+      </c>
+      <c r="DH2" t="s">
+        <v>135</v>
+      </c>
+      <c r="DI2" t="s">
+        <v>108</v>
+      </c>
+      <c r="DJ2" t="s">
+        <v>105</v>
+      </c>
+      <c r="DK2" t="s">
+        <v>136</v>
+      </c>
+      <c r="DL2" t="s">
+        <v>108</v>
+      </c>
+      <c r="DM2" t="s">
+        <v>137</v>
+      </c>
+      <c r="DN2" t="s">
+        <v>138</v>
+      </c>
+      <c r="DO2" t="s">
+        <v>107</v>
+      </c>
+      <c r="DP2" t="s">
+        <v>108</v>
+      </c>
+      <c r="DQ2" t="s">
+        <v>139</v>
+      </c>
+      <c r="DR2" t="s">
+        <v>140</v>
+      </c>
+      <c r="DS2" t="s">
+        <v>141</v>
+      </c>
+      <c r="DT2" t="s">
+        <v>142</v>
+      </c>
+      <c r="DU2" t="s">
+        <v>143</v>
+      </c>
+      <c r="DV2" t="s">
+        <v>144</v>
+      </c>
+      <c r="DW2" t="s">
         <v>145</v>
       </c>
-      <c r="CU2" t="s">
-        <v>122</v>
-      </c>
-      <c r="CV2" t="s">
-        <v>132</v>
-      </c>
-      <c r="CW2" t="s">
-        <v>123</v>
-      </c>
-      <c r="CX2" t="s">
-        <v>123</v>
-      </c>
-      <c r="CY2" t="s">
-        <v>132</v>
-      </c>
-      <c r="CZ2" t="s">
+      <c r="DX2" t="s">
+        <v>105</v>
+      </c>
+      <c r="DY2" t="s">
         <v>146</v>
-      </c>
-      <c r="DA2" t="s">
-        <v>147</v>
-      </c>
-      <c r="DB2" t="s">
-        <v>123</v>
-      </c>
-      <c r="DC2" t="s">
-        <v>123</v>
-      </c>
-      <c r="DD2" t="s">
-        <v>123</v>
-      </c>
-      <c r="DE2" t="s">
-        <v>123</v>
-      </c>
-      <c r="DF2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DG2" t="s">
-        <v>148</v>
-      </c>
-      <c r="DH2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DI2" t="s">
-        <v>149</v>
-      </c>
-      <c r="DJ2" t="s">
-        <v>149</v>
-      </c>
-      <c r="DK2" t="s">
-        <v>150</v>
-      </c>
-      <c r="DL2" t="s">
-        <v>151</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>152</v>
-      </c>
-      <c r="DO2" t="s">
-        <v>153</v>
-      </c>
-      <c r="DP2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DQ2" t="s">
-        <v>154</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>156</v>
-      </c>
-      <c r="DT2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DU2" t="s">
-        <v>157</v>
-      </c>
-      <c r="DV2" t="s">
-        <v>149</v>
-      </c>
-      <c r="DW2" t="s">
-        <v>148</v>
-      </c>
-      <c r="DX2" t="s">
-        <v>158</v>
-      </c>
-      <c r="DY2" t="s">
-        <v>132</v>
-      </c>
-      <c r="DZ2" t="s">
-        <v>158</v>
-      </c>
-      <c r="EA2" t="s">
-        <v>159</v>
-      </c>
-      <c r="EB2" t="s">
-        <v>132</v>
-      </c>
-      <c r="EC2" t="s">
-        <v>126</v>
-      </c>
-      <c r="ED2" t="s">
-        <v>160</v>
-      </c>
-      <c r="EE2" t="s">
-        <v>132</v>
-      </c>
-      <c r="EF2" t="s">
-        <v>161</v>
-      </c>
-      <c r="EG2" t="s">
-        <v>162</v>
-      </c>
-      <c r="EH2" t="s">
-        <v>129</v>
-      </c>
-      <c r="EI2" t="s">
-        <v>132</v>
-      </c>
-      <c r="EJ2" t="s">
-        <v>163</v>
-      </c>
-      <c r="EK2" t="s">
-        <v>164</v>
-      </c>
-      <c r="EL2" t="s">
-        <v>165</v>
-      </c>
-      <c r="EM2" t="s">
-        <v>166</v>
-      </c>
-      <c r="EN2" t="s">
-        <v>167</v>
-      </c>
-      <c r="EO2" t="s">
-        <v>168</v>
-      </c>
-      <c r="EP2" t="s">
-        <v>169</v>
-      </c>
-      <c r="EQ2" t="s">
-        <v>126</v>
-      </c>
-      <c r="ER2" t="s">
-        <v>170</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="45">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 DB2:DE2 AW2 AZ2:BD2 BK2 BO2 BQ2 BS2 BU2 CU2 CW2:CX2 K2:X2 Z2 AE2:AF2 AR2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="38">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2 CI2:CL2 AU2:AY2 CB2 CD2:CE2 K2:X2 Z2 AE2:AF2 AR2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AY2 CD2 EM2 EP2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2 CE2 CH2 CK2 CM2 CS2 CV2 CY2 DF2 DH2 DM2 DP2 DT2 DY2 EB2 EE2 EI2" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2 BK2 DT2 DW2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2 BL2 BO2 BR2 BT2 BZ2 CC2 CF2 CM2 CO2 CT2 CW2 DA2 DF2 DI2 DL2 DP2" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AZ2:BA2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2 AJ2:AK2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2 AJ2:AK2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2 AL2:AM2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2 AL2:AM2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2 AN2:AO2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2 AN2:AO2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J2 CZ2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J2 CG2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DR2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ED2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DK2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EF2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DM2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EG2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DN2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EH2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DO2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EJ2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EK2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DR2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DS2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EN2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DV2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-000021000000}">
-      <formula1>"Berdiri,Telentang"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000022000000}">
-      <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000023000000}">
-      <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BB2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Sudah,Belum"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BN2 BP2 BR2 BT2" xr:uid="{00000000-0002-0000-0000-000026000000}">
-      <formula1>"Positif,Negatif"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2" xr:uid="{00000000-0002-0000-0000-000027000000}">
-      <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-000028000000}">
-      <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-000029000000}">
-      <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2" xr:uid="{A76BCFDA-99B4-BC4C-9EB2-288C4CC41003}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">

</xml_diff>

<commit_message>
fix: stage 7 fixing skrining-filtering, doing modification for excel remaja and remaja.py
</commit_message>
<xml_diff>
--- a/dataset/remaja.xlsx
+++ b/dataset/remaja.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532CE790-9147-2141-A75A-B7E942522C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9979EDC3-0B54-8A4F-BFBD-CDA776052756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="-21000" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3300" yWindow="-21000" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -100,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="AP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -115,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="BK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -130,7 +130,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="BN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -145,7 +145,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -160,7 +160,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="BV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -180,7 +180,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="109">
   <si>
     <t>batas_awal</t>
   </si>
@@ -471,6 +471,42 @@
   </si>
   <si>
     <t>skrining_risiko_tb_anak</t>
+  </si>
+  <si>
+    <t>skrining_gizi</t>
+  </si>
+  <si>
+    <t>skrining_tekanan_darah_anak_remaja</t>
+  </si>
+  <si>
+    <t>skrining_gula_darah_anak</t>
+  </si>
+  <si>
+    <t>skrining_telinga_mata_anak_sekolah</t>
+  </si>
+  <si>
+    <t>skrining_tb_anak</t>
+  </si>
+  <si>
+    <t>skrining_frambusia</t>
+  </si>
+  <si>
+    <t>skrining_kusta</t>
+  </si>
+  <si>
+    <t>skrining_skabies</t>
+  </si>
+  <si>
+    <t>skrining_periksa_gigi_anak</t>
+  </si>
+  <si>
+    <t>skrining_hepatitis_b_7_12</t>
+  </si>
+  <si>
+    <t>skrining_rdt_malaria</t>
+  </si>
+  <si>
+    <t>skrining_risiko_tb</t>
   </si>
 </sst>
 </file>
@@ -898,7 +934,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CB5"/>
+  <dimension ref="A1:CM5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -922,37 +958,54 @@
     <col min="27" max="30" width="13" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="13" style="5" customWidth="1"/>
     <col min="32" max="33" width="13" customWidth="1"/>
-    <col min="34" max="37" width="14.33203125" customWidth="1"/>
-    <col min="38" max="38" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="4.1640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="24.1640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="44" width="24.1640625" customWidth="1"/>
-    <col min="45" max="45" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="46" max="51" width="24.1640625" customWidth="1"/>
-    <col min="52" max="52" width="14.33203125" customWidth="1"/>
-    <col min="53" max="53" width="25" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="59" max="60" width="14.83203125" customWidth="1"/>
-    <col min="61" max="61" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="22.83203125" customWidth="1"/>
-    <col min="65" max="65" width="16.1640625" customWidth="1"/>
-    <col min="66" max="66" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="67" max="68" width="12.33203125" customWidth="1"/>
-    <col min="69" max="69" width="14.1640625" customWidth="1"/>
-    <col min="70" max="70" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="16.1640625" customWidth="1"/>
+    <col min="34" max="34" width="14.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="14.33203125" customWidth="1"/>
+    <col min="37" max="37" width="32.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="14.33203125" customWidth="1"/>
+    <col min="40" max="40" width="22.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="31.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="48" width="24.1640625" customWidth="1"/>
+    <col min="49" max="49" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="55" width="24.1640625" customWidth="1"/>
+    <col min="56" max="56" width="20.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="25" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="14.83203125" customWidth="1"/>
+    <col min="64" max="64" width="14.83203125" style="5" customWidth="1"/>
+    <col min="65" max="65" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="22.83203125" customWidth="1"/>
+    <col min="69" max="69" width="22.83203125" style="5" customWidth="1"/>
+    <col min="70" max="70" width="16.1640625" customWidth="1"/>
+    <col min="71" max="71" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="19.83203125" style="5" customWidth="1"/>
+    <col min="73" max="74" width="12.33203125" customWidth="1"/>
+    <col min="75" max="75" width="14.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="14.1640625" customWidth="1"/>
+    <col min="77" max="77" width="14.1640625" style="5" customWidth="1"/>
+    <col min="78" max="78" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="16.5" style="5" customWidth="1"/>
+    <col min="80" max="80" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="16.1640625" style="5" customWidth="1"/>
+    <col min="82" max="82" width="16.1640625" customWidth="1"/>
+    <col min="83" max="83" width="16.1640625" style="5" customWidth="1"/>
+    <col min="84" max="84" width="25" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:80" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:91" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1050,144 +1103,182 @@
         <v>24</v>
       </c>
       <c r="AG1" s="2"/>
-      <c r="AH1" s="3" t="s">
+      <c r="AH1" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AI1" s="3" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AJ1" s="4" t="s">
+      <c r="AK1" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="AL1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="AK1" s="4" t="s">
+      <c r="AM1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="AL1" s="4" t="s">
+      <c r="AN1" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="AO1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AM1" s="4" t="s">
+      <c r="AP1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="AN1" s="4" t="s">
+      <c r="AQ1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="AO1" s="4" t="s">
+      <c r="AR1" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="AS1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="AP1" s="4" t="s">
+      <c r="AT1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AQ1" s="4" t="s">
+      <c r="AU1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="AR1" s="4" t="s">
+      <c r="AV1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="AS1" s="4" t="s">
+      <c r="AW1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AT1" s="4" t="s">
+      <c r="AX1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AU1" s="4" t="s">
+      <c r="AY1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AV1" s="4" t="s">
+      <c r="AZ1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AW1" s="4" t="s">
+      <c r="BA1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AX1" s="4" t="s">
+      <c r="BB1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AY1" s="4" t="s">
+      <c r="BC1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AZ1" s="2"/>
-      <c r="BA1" s="3" t="s">
+      <c r="BD1" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="BE1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BK1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="BI1" s="3" t="s">
+      <c r="BL1" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="BM1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="BJ1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="BK1" s="3" t="s">
+      <c r="BO1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="BL1" s="3" t="s">
+      <c r="BP1" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="BM1" s="3" t="s">
+      <c r="BQ1" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="BR1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="BN1" s="3" t="s">
+      <c r="BS1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="BO1" s="3" t="s">
+      <c r="BT1" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="BU1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="BP1" s="3" t="s">
+      <c r="BV1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="BQ1" s="3" t="s">
+      <c r="BW1" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="BX1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="BR1" s="3" t="s">
+      <c r="BY1" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="BZ1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="BS1" s="3" t="s">
+      <c r="CA1" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="CB1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="BT1" s="3" t="s">
+      <c r="CC1" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="CD1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CE1" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="CF1" t="s">
         <v>42</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CG1" t="s">
         <v>43</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CH1" t="s">
         <v>44</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CI1" t="s">
         <v>61</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CJ1" t="s">
         <v>46</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CK1" t="s">
         <v>47</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CL1" t="s">
         <v>62</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CM1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:80" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:91" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>64</v>
       </c>
@@ -1281,140 +1372,176 @@
       <c r="AF2" t="s">
         <v>69</v>
       </c>
-      <c r="AH2">
+      <c r="AH2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI2">
         <v>50</v>
       </c>
-      <c r="AI2">
+      <c r="AJ2">
         <v>130</v>
       </c>
-      <c r="AJ2">
+      <c r="AK2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL2">
         <v>120</v>
       </c>
-      <c r="AK2">
+      <c r="AM2">
         <v>80</v>
       </c>
-      <c r="AL2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN2">
+      <c r="AN2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ2">
         <v>120</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AR2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AS2" t="s">
         <v>70</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AT2" t="s">
         <v>70</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AU2" t="s">
         <v>71</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AV2" t="s">
         <v>71</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AW2" t="s">
         <v>72</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AX2" t="s">
         <v>72</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AY2" t="s">
         <v>70</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AZ2" t="s">
         <v>70</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="BA2" t="s">
         <v>73</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="BB2" t="s">
         <v>73</v>
       </c>
-      <c r="AY2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA2" t="s">
+      <c r="BC2" t="s">
+        <v>67</v>
+      </c>
+      <c r="BD2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BE2" t="s">
         <v>69</v>
       </c>
-      <c r="BB2" t="s">
-        <v>68</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>68</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>68</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>68</v>
-      </c>
       <c r="BF2" t="s">
         <v>68</v>
       </c>
       <c r="BG2" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>68</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ2" t="s">
+        <v>68</v>
+      </c>
+      <c r="BK2" t="s">
         <v>70</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BL2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BM2" t="s">
         <v>74</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BN2" t="s">
         <v>75</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BO2" t="s">
         <v>76</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BP2" t="s">
         <v>77</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BQ2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR2" t="s">
         <v>78</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BS2" t="s">
         <v>79</v>
       </c>
-      <c r="BO2" t="s">
+      <c r="BT2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BU2" t="s">
         <v>80</v>
       </c>
-      <c r="BP2" t="s">
+      <c r="BV2" t="s">
         <v>81</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BX2" t="s">
         <v>82</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="BY2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BZ2" t="s">
         <v>83</v>
       </c>
-      <c r="BS2" t="s">
+      <c r="CA2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CB2" t="s">
         <v>84</v>
       </c>
-      <c r="BT2" t="s">
+      <c r="CC2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CD2" t="s">
         <v>85</v>
       </c>
-      <c r="BU2" t="s">
+      <c r="CE2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CF2" t="s">
         <v>69</v>
       </c>
-      <c r="BV2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BY2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BZ2" t="s">
-        <v>67</v>
-      </c>
-      <c r="CA2" t="s">
+      <c r="CG2" t="s">
+        <v>67</v>
+      </c>
+      <c r="CH2" t="s">
+        <v>67</v>
+      </c>
+      <c r="CI2" t="s">
+        <v>67</v>
+      </c>
+      <c r="CJ2" t="s">
+        <v>67</v>
+      </c>
+      <c r="CK2" t="s">
+        <v>67</v>
+      </c>
+      <c r="CL2" t="s">
         <v>69</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CM2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:80" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:91" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>87</v>
       </c>
@@ -1508,203 +1635,275 @@
       <c r="AF3" t="s">
         <v>69</v>
       </c>
-      <c r="AH3">
+      <c r="AH3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI3">
         <v>50</v>
       </c>
-      <c r="AI3">
+      <c r="AJ3">
         <v>130</v>
       </c>
-      <c r="AJ3">
+      <c r="AK3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AL3">
         <v>120</v>
       </c>
-      <c r="AK3">
+      <c r="AM3">
         <v>80</v>
       </c>
-      <c r="AL3" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN3">
+      <c r="AN3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ3">
         <v>120</v>
       </c>
-      <c r="AO3" t="s">
+      <c r="AR3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AS3" t="s">
         <v>70</v>
       </c>
-      <c r="AP3" t="s">
+      <c r="AT3" t="s">
         <v>70</v>
       </c>
-      <c r="AQ3" t="s">
+      <c r="AU3" t="s">
         <v>71</v>
       </c>
-      <c r="AR3" t="s">
+      <c r="AV3" t="s">
         <v>71</v>
       </c>
-      <c r="AS3" t="s">
+      <c r="AW3" t="s">
         <v>72</v>
       </c>
-      <c r="AT3" t="s">
+      <c r="AX3" t="s">
         <v>72</v>
       </c>
-      <c r="AU3" t="s">
+      <c r="AY3" t="s">
         <v>70</v>
       </c>
-      <c r="AV3" t="s">
+      <c r="AZ3" t="s">
         <v>70</v>
       </c>
-      <c r="AW3" t="s">
+      <c r="BA3" t="s">
         <v>73</v>
       </c>
-      <c r="AX3" t="s">
+      <c r="BB3" t="s">
         <v>73</v>
       </c>
-      <c r="AY3" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA3" t="s">
+      <c r="BC3" t="s">
+        <v>67</v>
+      </c>
+      <c r="BD3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BE3" t="s">
         <v>69</v>
       </c>
-      <c r="BB3" t="s">
-        <v>68</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>68</v>
-      </c>
-      <c r="BD3" t="s">
-        <v>68</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>68</v>
-      </c>
       <c r="BF3" t="s">
         <v>68</v>
       </c>
       <c r="BG3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BH3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BK3" t="s">
         <v>70</v>
       </c>
-      <c r="BI3" t="s">
+      <c r="BL3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BM3" t="s">
         <v>74</v>
       </c>
-      <c r="BJ3" t="s">
+      <c r="BN3" t="s">
         <v>75</v>
       </c>
-      <c r="BK3" t="s">
+      <c r="BO3" t="s">
         <v>76</v>
       </c>
-      <c r="BL3" t="s">
+      <c r="BP3" t="s">
         <v>77</v>
       </c>
-      <c r="BM3" t="s">
+      <c r="BQ3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR3" t="s">
         <v>78</v>
       </c>
-      <c r="BN3" t="s">
+      <c r="BS3" t="s">
         <v>79</v>
       </c>
-      <c r="BO3" t="s">
+      <c r="BT3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BU3" t="s">
         <v>80</v>
       </c>
-      <c r="BP3" t="s">
+      <c r="BV3" t="s">
         <v>81</v>
       </c>
-      <c r="BQ3" t="s">
+      <c r="BX3" t="s">
         <v>82</v>
       </c>
-      <c r="BR3" t="s">
+      <c r="BY3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BZ3" t="s">
         <v>83</v>
       </c>
-      <c r="BS3" t="s">
+      <c r="CA3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CB3" t="s">
         <v>84</v>
       </c>
-      <c r="BT3" t="s">
+      <c r="CC3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CD3" t="s">
         <v>85</v>
       </c>
-      <c r="BU3" t="s">
+      <c r="CE3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CF3" t="s">
         <v>69</v>
       </c>
-      <c r="BV3" t="s">
-        <v>67</v>
-      </c>
-      <c r="BW3" t="s">
-        <v>67</v>
-      </c>
-      <c r="BX3" t="s">
-        <v>67</v>
-      </c>
-      <c r="BY3" t="s">
-        <v>67</v>
-      </c>
-      <c r="BZ3" t="s">
-        <v>67</v>
-      </c>
-      <c r="CA3" t="s">
+      <c r="CG3" t="s">
+        <v>67</v>
+      </c>
+      <c r="CH3" t="s">
+        <v>67</v>
+      </c>
+      <c r="CI3" t="s">
+        <v>67</v>
+      </c>
+      <c r="CJ3" t="s">
+        <v>67</v>
+      </c>
+      <c r="CK3" t="s">
+        <v>67</v>
+      </c>
+      <c r="CL3" t="s">
         <v>69</v>
       </c>
-      <c r="CB3" t="s">
+      <c r="CM3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:80" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:91" x14ac:dyDescent="0.2">
       <c r="D4" s="6"/>
+      <c r="AH4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AK4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AR4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BD4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BL4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BQ4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BT4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="BY4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CA4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CC4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="CE4" s="5" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="5" spans="1:80" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:91" x14ac:dyDescent="0.2">
       <c r="D5" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="20">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3 AG2:AG3 AL2:AM3 AY2:AY3 BB2:BF3 BV2:BZ3 D2:D5 K2:AE3" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3 K2:AE3 AO2:AP3 BC2:BC3 BF2:BJ3 CG2:CK3 D2:D5 AG2:AG3 AH2:AH4 AK2:AK4 AN2:AN4 AR2:AR4 BD2:BD4 BL2:BL4 BQ2:BQ4 BT2:BT4 BY2:BY4 CA2:CA4 CC2:CC4 CE2:CE4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AF2:AF3 BA2:BA3 BL2:BL3 BU2:BU3 CA2:CA3" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2:BH3" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AF2:AF3 BE2:BE3 CL2:CL3 CF2:CF3 BP2:BP3" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2:BK3" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI3" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2:BM3" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ2:BJ3" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2:BN3" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2:BK3" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2:BO3" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2:BM3" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2:BR3" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2:BN3" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2:BS3" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2:BO3" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU3" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2:BP3" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2:BV3" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2:BQ3" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BY3 CA2:CA3 CC2:CC3 CE2:CE3" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AR3" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AV3" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2:AT3" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2:AX3" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AV3" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AY2:AZ3" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:J3" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2:BS3" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB3" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2:BR3" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2:BZ3" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2:AP3" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2:AT3" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal,Ada indikasi gangguan pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2:AX3" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2:BB3" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Normal (visus 6/6 - 6/9),Ada indikasi gangguan penglihatan (visus &lt;6/9)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2:BT3" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2:CD3" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Reaktif,Non-Reaktif"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>